<commit_message>
Quarterly scrape (Medium): Q2 2026
</commit_message>
<xml_diff>
--- a/GOWT_mid_low.xlsx
+++ b/GOWT_mid_low.xlsx
@@ -41354,7 +41354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -43403,6 +43403,1815 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>CoolDrive</t>
+        </is>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>CoolDrive Expands Battery Offerings with VARTA (18/05/2026)
+CoolDrive Auto Parts expanded its product range by introducing the globally recognised VARTA automotive battery line, signaling continued growth in its automotive aftermarket offering and product portfolio.
+CoolDrive Breaks Ground on New Head Office and Distribution Centre (23/10/2025)
+CoolDrive Auto Parts began construction on a new head office and national distribution centre in Boronia, Victoria. The project will consolidate three Melbourne distribution centres into one larger, more automated facility, improving logistics efficiency and supporting future growth.
+Success for CoolDrive at the AAAE (23/04/2024)
+CoolDrive showcased its products at the 2024 Australian Auto Aftermarket Expo and won an Auto Aftermarket Excellence Award for the GYS Powerduction 37LG. The event highlighted the company’s strong industry presence and ongoing momentum.</t>
+        </is>
+      </c>
+      <c r="D71" s="17" t="inlineStr">
+        <is>
+          <t>[19/05/2026 - today] Opening of CoolDrive's second South Australian branch in Melrose Park for improved delivery service.
+[18/05/2026 - 1d] John Blanchard recognized with the Outstanding Service to Industry Award at the awards ceremony.
+[16/05/2026 - 3d] Recap of the expo week and mentions of multiple awards won by CoolDrive.
+[15/05/2026 - 4d] Recognition at the Australian Auto Aftermarket Expo for winning Best Stand over 36m2.</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/cooldrive-distribution/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>Corporate Protection</t>
+        </is>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="C72" s="17" t="inlineStr">
+        <is>
+          <t>Corporate Protection positions itself as Australia’s largest privately owned emergency services company (01/01/2024)
+Corporate Protection’s corporate website states that the business is Australia’s largest privately owned emergency services company, highlighting its scale and sustained business growth over more than 25 years in operation.
+Corporate Protection expands international services across Southeast Asia and the Pacific Rim (01/01/2007)
+Corporate Protection announced the establishment of Corporate Protection International (CPI) in 2007 to serve international demand with a broader suite of services, including induction, medical, emergency response, security, training, and consultancy across Southeast Asia and the Pacific Rim. This indicates geographic and service-line expansion for the Brisbane-headquartered company.</t>
+        </is>
+      </c>
+      <c r="D72" s="17" t="inlineStr">
+        <is>
+          <t>[19/05/2026 - today] Corporate Protection is hiring for leadership roles in Maritime Security, indicating expansion of their team and service offerings.
+[18/05/2026 - 1d] Corporate Protection announces a new hiring opportunity for a Paramedic in Brisbane, indicating team growth.
+[18/05/2026 - 1d] Corporate Protection announces another hiring opportunity for a Paramedic, further signifying ongoing recruitment efforts.</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/corporate-protection/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>CoverTel Telecommunications Group</t>
+        </is>
+      </c>
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>CoverTel and Phase Pacific join forces to accelerate growth and expand customer reach (01/03/2024)
+CoverTel Telecommunications Group announced a strategic collaboration with Phase Pacific, a Melbourne-based company specialising in network integrity, software integrity and automation. The partnership aims to accelerate Phase Pacific’s growth while enabling CoverTel to explore new customer segments and broaden its market reach by combining complementary product portfolios and technical capabilities. The collaboration underscores CoverTel’s expansion strategy in advanced test, measurement, and network solutions for telecommunications and related industries.
+Phase Pacific and CoverTel join forces to enhance network solutions across Australia (01/03/2024)
+In a joint announcement, Phase Pacific and CoverTel Telecommunications Group detailed their new strategic partnership focused on delivering enhanced network solutions. CoverTel, founded in 2002 and headquartered in Melbourne, will leverage its established presence across sectors such as Oil, Mining, Gas, Rail, Energy, Utilities, Defence, IT and Telecom to extend the reach of Phase Pacific’s network integrity and automation offerings. The collaboration is positioned as a growth initiative for both companies, strengthening CoverTel’s solution portfolio and reinforcing its role as a leading telecommunications solutions provider in Australia.
+CoverTel continues multi‑sector expansion as a trusted supplier of telecoms and network solutions (01/01/2024)
+CoverTel highlights ongoing growth as a trusted supplier to major Telecommunications and Utility providers across Australia and the Pacific Islands, reflecting more than 20 years of continuous expansion. The company notes that its extensive product portfolio has enabled it to grow beyond core telecommunications into Defence, Data Centres and Enterprise markets. This diversification into new verticals and broader infrastructure, monitoring, and test-and-measurement offerings signals sustained business expansion and a strengthening market position for the Melbourne‑headquartered firm.</t>
+        </is>
+      </c>
+      <c r="D73" s="17" t="inlineStr"/>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/covertel-telecommunications-group/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>Customer Radar</t>
+        </is>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
+        <is>
+          <t>Auckland</t>
+        </is>
+      </c>
+      <c r="C74" s="17" t="inlineStr">
+        <is>
+          <t>What customer feedback tells us (04/11/2015)
+Customer Radar announces it has captured its one‑millionth piece of customer feedback in five years, with more than 1,000 active feedback ‘measures’ (stores, departments or people) on the platform. Founder Mat Wylie notes that, based on accelerating uptake, the next million responses are expected in under 12 months. The company also signals plans to expand beyond New Zealand into Australasia and other English‑speaking markets, underscoring strong user growth and international expansion ambitions.
+'Customer radar' in real time (17/09/2013)
+Interest.co.nz profiles Customer Radar’s cloud‑based real‑time customer feedback software as a disruptive alternative to traditional market research. The piece details how the platform provides live dashboards and alerting for negative feedback, enabling quicker service recovery and better decision‑making for client businesses. The coverage raises the company’s profile in the business support services and SaaS sectors and signals market traction for its technology.
+Radar homes in on customers (02/07/2013)
+Profile of Auckland-based Customer Radar, founded by advertising executive Mat Wylie, describing how the company’s real‑time feedback platform is enabling businesses to capture customer opinions via text and web apps. The article highlights the firm’s technology-driven shift from a traditional advertising background into scalable business support services, positioning Customer Radar for growth in the customer experience and feedback analytics market.</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="inlineStr"/>
+      <c r="E74" s="16" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>Cyber Risk</t>
+        </is>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C75" s="17" t="inlineStr"/>
+      <c r="D75" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Collaboration with Serena Williams and Reckitt to empower underrepresented founders and build networks.
+[27/04/2026 - 3w] LinkedIn is the most-cited domain on AI search engines, indicating growth in professional visibility.
+[22/04/2026 - 3w] Announcement of new leadership roles within LinkedIn, indicating growth and opportunity.</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>Dan Smethurst Orthodontist</t>
+        </is>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="inlineStr">
+        <is>
+          <t>Dan Smethurst Orthodontist Recognised as Diamond Invisalign® Provider in Tauranga (01/03/2023)
+Dan Smethurst Orthodontist has been recognised as a Diamond Invisalign® provider, reflecting a very high volume of completed Invisalign cases and strong clinical expertise. The status—highlighted on the practice’s Invisalign-focused pages and patient success materials—indicates sustained growth in clear-aligner treatments and positions the clinic as a leading provider in Tauranga and the Bay of Plenty region.
+Remote Dental Monitoring Service Introduced to Support Invisalign Growth at Dan Smethurst Orthodontist (15/06/2022)
+Dan Smethurst Orthodontist has implemented Dental Monitoring, a smartphone-based remote orthodontic tracking system, to support its expanding Invisalign patient base. By allowing the specialist orthodontist to review progress more frequently without in-person visits, the practice increases capacity, improves convenience for patients, and enhances its digital-care capabilities—signs of operational and service expansion.
+Dan Smethurst Orthodontist Highlights Hundreds of Successful Invisalign Cases in Tauranga and Bay of Plenty (10/10/2021)
+Through its ‘Patient Success’ and ‘Before and After’ galleries, Dan Smethurst Orthodontist showcases hundreds of completed Invisalign and orthodontic treatments from Tauranga and the wider Bay of Plenty. The volume of documented cases and testimonials points to strong and sustained patient demand, underpinning the practice’s growth and reinforcing its reputation as a leading orthodontic provider in the region.</t>
+        </is>
+      </c>
+      <c r="D76" s="17" t="inlineStr"/>
+      <c r="E76" s="16" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t>Darzin Software Pty Ltd</t>
+        </is>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="inlineStr">
+        <is>
+          <t>Darzin highlighted as Australia’s trusted name in stakeholder engagement software with global customer base (01/06/2021)
+Darzin describes itself as Australia’s trusted name in stakeholder engagement software, now serving customers around the world with a team of developers, designers, information architects, UX specialists, business analysts, engineers and testers. The emphasis on an expanded multidisciplinary team and global clients indicates sustained growth in headcount and market reach since its founding in 2004.
+Darzin profiled as growing SaaS employer with 11–50 staff (01/05/2021)
+Startup and tech‑employer directory Matchstiq lists Darzin as a Sydney‑based SaaS company with 11–50 employees and positions it as Australia’s trusted name in stakeholder relationship management. The profile underscores the company’s evolution from a small founder‑led business in 2004 to a larger, established SaaS employer with growing staff numbers and ongoing hiring needs.
+Darzin recognised as feature‑rich, easy‑to‑use stakeholder engagement platform with clients across the globe (01/03/2021)
+Industry review site FeaturedCustomers profiles Darzin as one of the most feature‑rich and easy‑to‑use stakeholder engagement platforms on the market, noting that the company has clients across the globe. The recognition and international customer base point to product maturity, market traction and ongoing commercial growth for the Sydney‑based software company.
+Simply Stakeholders brand becomes parent company, expanding beyond original Darzin product (01/04/2020)
+Simply Stakeholders (the parent company founded around the original Darzin product) now positions Darzin as its original stakeholder engagement platform while building a broader global suite of stakeholder software. This signals growth from a single-product firm into a multi‑product, global stakeholder software company, highlighting expansion in product scope and international reach.</t>
+        </is>
+      </c>
+      <c r="D77" s="17" t="inlineStr"/>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/darzin-software/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="16" t="inlineStr">
+        <is>
+          <t>Data Capture Experts</t>
+        </is>
+      </c>
+      <c r="B78" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C78" s="17" t="inlineStr">
+        <is>
+          <t>Data Capture Experts Announces Three New Appointments to Board of Directors (22/04/2024)
+Melbourne-based Data Capture Experts, a fast-growing healthcare technology company, appointed three new board directors—Vicki Gillespie (as Chair), John Papatheohari and Andrew Harris—to accelerate growth, innovation and geographic expansion of its DC2Vue digital health platform across Australia and beyond.
+Data Capture Experts Appoints Danny Lindrea as Chief Digital Health Officer (28/11/2023)
+Data Capture Experts strengthened its executive leadership team by appointing experienced digital health leader Danny Lindrea as Chief Digital Health Officer, supporting the company’s strategy to scale its next-generation DC2Vue care coordination platform and advance connected healthcare.</t>
+        </is>
+      </c>
+      <c r="D78" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Announcement of a partnership with Serena Williams and Reckitt to support underrepresented founders and emphasize the importance of networking.
+[27/04/2026 - 3w] Information about LinkedIn being the most cited domain for professional queries, indicating growth in market presence.
+[22/04/2026 - 3w] Announcement of new leadership positions at LinkedIn, indicating future opportunities for growth.</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>DataTorque</t>
+        </is>
+      </c>
+      <c r="B79" s="16" t="inlineStr">
+        <is>
+          <t>Wellington</t>
+        </is>
+      </c>
+      <c r="C79" s="17" t="inlineStr">
+        <is>
+          <t>TIN Member Spotlight highlights DataTorque’s rapid revenue growth and $60m in new contracts (15/09/2023)
+Technology Investment Network’s member spotlight on DataTorque reports that the Wellington‑headquartered tax and revenue management software company has appeared four times on TIN’s Absolute IT Supreme Scale-Ups list. The article notes 26% revenue growth since 2020 and more than NZ$60m in contracts signed since 2018, reflecting strong international expansion of its Commercial Off‑the‑Shelf Revenue Management System, now deployed to support tax collection in 16 countries across the Pacific, Africa, the Americas and Europe.
+Private equity investment by Simplicity backs DataTorque’s next growth phase (09/03/2023)
+Law firm MinterEllisonRuddWatts advised Wellington-based DataTorque on selling a minority stake to the private equity fund of Simplicity, a major New Zealand non‑profit KiwiSaver and investment fund manager. The investment is positioned as growth capital to help the company scale its leading tax technology and revenue management solutions, which already support more efficient public revenue collection in 16 countries worldwide.
+DataTorque profiled as fintech transforming economies with people‑centred digital tax systems (10/11/2022)
+A See Tomorrow First profile describes Wellington-based fintech DataTorque as transforming economies by engineering people‑centred digital solutions for public revenue collection. The article emphasises the company’s growing global footprint and role in modernising tax systems for governments, reinforcing its reputation and positioning that support further international expansion.</t>
+        </is>
+      </c>
+      <c r="D79" s="17" t="inlineStr"/>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/data-doctors-nz-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>Datarwe</t>
+        </is>
+      </c>
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="C80" s="17" t="inlineStr">
+        <is>
+          <t>Datarwe acknowledged as exemplar in AI-enabled healthcare industry report (01/09/2022)
+Datarwe was highlighted as the exemplar in a major publication on AI-enabled healthcare, recognised for its precision data platform that underpins development of AI clinical diagnostic tools. The report showcases Datarwe as one of nine knowledge-based emerging seed industries in Queensland, reinforcing its leadership position and supporting future growth and investment opportunities.
+Datarwe relocates HQ to Gold Coast Health &amp; Knowledge Precinct and scales AI healthcare platform (04/02/2022)
+A Lumina/Gold Coast Health &amp; Knowledge Precinct case study notes that Datarwe, founded in 2019, rapidly expanded after relocating its headquarters to the Precinct in 2020. The company’s precision medicine data platform is being rolled out to 14 Queensland hospital sites, with national and international deployments in the pipeline, and is involved in a high‑profile collaboration with MIT on the MIMIC critical care database—highlighting expansion, partnerships and market traction.
+Datarwe collaborates with Queensland Health on Nursing Acuity Dashboard (01/10/2021)
+Datarwe’s website highlights a collaboration with Queensland Health to develop a Nursing Acuity Dashboard that uses real‑world ICU data to improve workflow efficiency. The project demonstrates increased adoption of Datarwe’s AI-driven data service platform within the public health system and broadens its solution portfolio for acute care environments.
+Datarwe opens new AI lab within Cohort at Gold Coast Health &amp; Knowledge Precinct (15/03/2021)
+Datarwe announced the opening of a dedicated AI lab within the Cohort Innovation Space at the Gold Coast Health &amp; Knowledge Precinct. The facility is designed to support collaborative R&amp;D with clinicians, researchers, and industry partners, expanding Datarwe’s physical footprint and R&amp;D capacity in AI-enabled healthcare data services.
+Datarwe launches Clinical Data Nexus to connect hospitals and med‑tech innovators (01/11/2020)
+The Queensland AI Hub profiled Datarwe’s launch of its Clinical Data Nexus (CDN) in late 2020, a curated and enriched real‑world clinical data platform for hospitals, clinicians, researchers, and AI/ML developers. The article highlights Datarwe’s rapid team growth to around 24 employees across Australia and WA and its role enabling faster, more cost‑effective AI‑enabled medical innovation—signalling both product and headcount expansion.
+KJR helps Datarwe build secure multi-layered clinical data access platform (01/06/2020)
+Technology consultancy KJR detailed its partnership with Datarwe to architect and deliver a secure, multi-layered data access platform for high-quality clinical data. The collaboration strengthened Datarwe’s core product—the clinical data-sharing platform that underpins AI models—representing a key strategic technology partnership supporting scalable growth.
+Datarwe receives $1.5M funding boost from Queensland Government (30/04/2020)
+The Queensland Government, through the Advance Queensland initiative, invested $1.5 million in Datarwe to accelerate development of its Precision Medicine Data Platform. The funding supports the company’s acute care medical research data platform that uses de-identified ICU data to enable AI-enabled clinical diagnostic tools, cementing Datarwe’s role as a key public‑private partner with Queensland Health and ecosystem partners like AWS, KJR and TechConnect.</t>
+        </is>
+      </c>
+      <c r="D80" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Collaboration with Serena Williams and Reckitt to enhance networking and support underrepresented founders.
+[22/04/2026 - 3w] Announcement of new leadership roles for Daniel Shapero and Mohak Shroff at LinkedIn, indicating organizational growth.</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>Delta Hydraulics (Tasmania, Australia)</t>
+        </is>
+      </c>
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>Tasmania</t>
+        </is>
+      </c>
+      <c r="C81" s="17" t="inlineStr">
+        <is>
+          <t>Prime Minister visits Delta Hydraulics’ Devonport plant after landmark energy MoU (15/12/2020)
+Following the signing of an energy supply memorandum of understanding between the Australian Prime Minister and the Tasmanian Premier, Prime Minister Scott Morrison visited Delta Hydraulics’ Devonport facility. The visit highlighted Delta Hydraulics as Australia’s largest independent hydraulic component manufacturer (established in 1975) and underscored the company’s importance to regional advanced manufacturing and future growth supported by secure energy supply.
+Industry profile: John White highlights resilience and innovation at Delta Hydraulics’ Devonport facility (01/03/2019)
+An industry feature on founder and Managing Director John White described Delta Hydraulics’ Devonport plant as central to ongoing innovation in hydraulic cylinder technology, including products like the Delta‑C cylinder designed to extend service life in harsh environments. White stressed that the resilience of the Tasmanian manufacturing base is crucial for supplying advanced products to Australian transport equipment manufacturers, reinforcing the company’s commitment to R&amp;D‑driven growth from its home facility.
+Merger consolidates Delta Hydraulics Group with White Hot Industries to drive growth (02/07/2018)
+Jason Bresnehan completed a merger of two related‑party businesses within the John White Group, bringing together Delta Hydraulics Group and White Hot Industries Group. The transaction consolidated Delta Hydraulics Pty Ltd in Devonport—described as a world‑leading manufacturer and innovator of telescopic and industrial hydraulic cylinders—with its related operations, aiming to create efficiencies, strengthen global supply to industries such as underground mining and transport, and support continued expansion from the Tasmanian base.
+Delta Hydraulics upgrades Tasmania factory to become high‑tech telescopic cylinder hub (01/09/2016)
+Delta Hydraulics invested approximately $2 million to upgrade its Devonport, Tasmania manufacturing facility, installing high‑tech skiving‑burnishing machines, friction welders, CNC lathes and CNC turning units. The upgrade supports a strategic shift: standard, off‑the‑shelf cylinder production has been moved to a newer Thailand factory, while the Tasmanian plant is positioned as the company’s specialised, value‑added manufacturing centre and an unofficial high‑tech telescopic cylinder hub for the Southern Hemisphere.
+Delta Hydraulics marks 40 years as Australia’s largest independent hydraulics manufacturer (01/06/2015)
+On its 40th anniversary, Delta Hydraulics was profiled as Australia’s largest independent maker of hydraulic components. The coverage emphasised the company’s long‑term growth from its Tasmanian origins into a major national and international supplier, with ongoing plans to pursue opportunities in Thailand and China, reflecting both sustained financial resilience and international expansion ambitions rooted in its Devonport operations.</t>
+        </is>
+      </c>
+      <c r="D81" s="17" t="inlineStr"/>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/delta-hydraulics-pty-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>DermCo</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>Perth</t>
+        </is>
+      </c>
+      <c r="C82" s="17" t="inlineStr"/>
+      <c r="D82" s="17" t="inlineStr"/>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/dermco-pty-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>DermEd (Brisbane, AU)</t>
+        </is>
+      </c>
+      <c r="B83" s="16" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="C83" s="17" t="inlineStr"/>
+      <c r="D83" s="17" t="inlineStr">
+        <is>
+          <t>[05/05/2026 - 2w] Dr Manoharan presents at Cutera University, highlighting partnerships and collaboration in education.
+[28/04/2026 - 3w] High interest in observership programs leads to opening more application slots, indicating team growth and demand.</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/dermed-laser-education/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="inlineStr">
+        <is>
+          <t>Diverseco</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>South Australia</t>
+        </is>
+      </c>
+      <c r="C84" s="17" t="inlineStr">
+        <is>
+          <t>Diverseco builds national presence in robotics, intralogistics and automation (01/03/2024)
+Positioning itself as an industry leader in robotics, intralogistics and automation, Diverseco reports over 30 years of growth built on cutting‑edge weighing and automation technologies along with maintenance and calibration services. The company emphasises that its products and services enable Australian companies to improve efficiency and scale through turnkey solutions. This ongoing evolution from a weighing-focused business into a broader automation and service provider demonstrates continued strategic growth in both capabilities and market positioning.
+Growth drives Diverseco rebrand (01/07/2016)
+Diverseco announced a major organisational rebrand to unify its portfolio companies – AccuWeigh, Robot Technologies-Systems Australia, AccuPak, AccuOnboard, SCACO and Ultrahawke – under the single Diverseco name. CEO Brenton Cunningham said the move was driven by a goal to grow the group from a mid-$40 million business to a $100 million business, and to create greater cohesion across its weighing, dimensional measurement, robotics automation, end‑of‑line packaging and product inspection operations. The rebrand coincided with the establishment of Diverseco South‑East Asia, based in Singapore, signalling international expansion ambitions.
+Diverseco expands through serial acquisitions in weighing and automation (01/01/2016)
+Diverseco’s history highlights sustained expansion in the machinery and equipment space via multiple acquisitions aligned to weighing and automation. Building on AccuWeigh’s growth – including being listed in BRW’s Fast 100 Companies in 2000 – the group acquired Ultrahawke in 2000, Queensland Weighing Machines in 2004, Independent Scales NZ and Budpak in 2006, Scale Components in 2009, Colonial Weighing in 2010, Sydney Weighbridges in 2015, and Robot Technologies Systems in 2016. These deals have broadened Diverseco’s geographic footprint across Australia and New Zealand and deepened its capabilities in weighbridges, industrial weighing, packaging and automation systems, reflecting a long‑term growth strategy.
+SCACO parent Diverseco acquires Robotic Technologies Australia as part of national expansion (01/12/2015)
+Diverseco, the parent company of SCACO, acquired Melbourne-based Robotic Technologies Australia, a leading robotics and automation business, as part of a broader national growth strategy built on targeted acquisitions. The purchase brought the number of acquisitions completed by managing director Brenton Cunningham to ten, following the acquisition of Sydney Weighbridges the previous year. With AccuWeigh remaining the core business and accounting for about half of group turnover, Diverseco’s annual revenue exceeded $40 million and was forecast to reach $45 million, underscoring strong financial and operational growth in its weighing, packaging and automation portfolio.</t>
+        </is>
+      </c>
+      <c r="D84" s="17" t="inlineStr">
+        <is>
+          <t>[14/05/2026 - 5d] Diverseco attended the unveiling of a new project by C2 Robotics, showcasing partnership and innovation in automation.
+[08/05/2026 - 1w] Diverseco revives Accuweigh as a dedicated brand for weighing solutions, emphasizing commitment to industry.
+[24/04/2026 - 3w] Diverseco announces completion of a weighbridge installation for City Circle Group, showcasing successful project execution.
+[23/04/2026 - 3w] Diverseco welcomes Paul Mason as the new CEO of Robotics Australia Group, indicating leadership stability.
+[20/04/2026 - 4w] Diverseco showcases their exhibit at the Robotics Expo, discussing future projects, including a 'Factory of the Future.'</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/diverseco/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="16" t="inlineStr">
+        <is>
+          <t>Dogcity Daycare (Adelaide, SA, Australia)</t>
+        </is>
+      </c>
+      <c r="B85" s="16" t="inlineStr">
+        <is>
+          <t>Adelaide</t>
+        </is>
+      </c>
+      <c r="C85" s="17" t="inlineStr">
+        <is>
+          <t>Dogcity Daycare continues metro expansion with new Ridgehaven centre (15/03/2023)
+Dogcity Daycare, Adelaide’s largest doggy daycare provider, has expanded beyond its original Kent Town headquarters by opening a new Ridgehaven location in Adelaide’s north-east. The Ridgehaven centre, listed at 6 Norma Avenue with dedicated contact details and booking portal, adds to existing sites in Kent Town, Thebarton, Keswick and Hampstead Gardens. This fifth site strengthens Dogcity’s metro footprint, increases capacity for daycare and grooming services, and reflects sustained demand for their force‑free, enrichment-focused daycare model.
+Dogcity Daycare grows to four-location network across Adelaide (18/06/2022)
+Lifestyle outlet Glam Adelaide profiled Dogcity Daycare’s growth to a four-site network—Hampstead Gardens (NORTH), Keswick (SOUTH), Kent Town (EAST) and Thebarton (WEST)—as part of coverage of an open day at the Kent Town facility. The article highlights Dogcity’s status as a leading doggy daycare provider in South Australia, notes strong customer demand reflected in discounted multi-visit packs, and emphasises that daycare credits are valid across all four locations, signalling operational scale and integrated services across metropolitan Adelaide.
+Dogcity Daycare builds leading position with multi-site operations and force‑free accreditation (01/12/2021)
+Dogcity Daycare’s own company information describes it as the largest and leading provider of doggy daycare in South Australia, supported by multiple locations (Kent Town, Thebarton, Keswick, Hampstead Gardens and later Ridgehaven), an International Force‑Free accreditation, custom indoor facilities, structured puppy socialisation programs, and value‑added offerings like lunch orders and birthday parties. While not a single news event, this profile evidences sustained growth through geographic expansion, service diversification, and professional accreditation in the recreational pet services sector.</t>
+        </is>
+      </c>
+      <c r="D85" s="17" t="inlineStr"/>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/dogcity-daycare/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="16" t="inlineStr">
+        <is>
+          <t>Dr Deb Harris, University Drive, Callaghan, Newcastle University, New South Wales 2308, AU</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="inlineStr">
+        <is>
+          <t>New South Wales</t>
+        </is>
+      </c>
+      <c r="C86" s="17" t="inlineStr">
+        <is>
+          <t>Professor Deborah Harris recognised as internationally recognised nursing and midwifery researcher (01/01/2026)
+Profile information from the University of Newcastle highlights Professor Deborah Harris’s standing as an internationally recognised researcher with expertise across neonatal care and the nurse practitioner workforce, indicating professional growth and recognition.
+Professor Deborah Harris profile highlights leadership in nursing and midwifery research (01/01/2026)
+The University of Newcastle profile notes Deborah Harris’s senior leadership and research expertise, including her role across nursing and midwifery research areas, suggesting continued professional advancement and institutional growth.</t>
+        </is>
+      </c>
+      <c r="D86" s="17" t="inlineStr">
+        <is>
+          <t>[14/05/2026 - 5d] An initiative by the Breathe 4 Bub program aimed at addressing asthma in Aboriginal women, showcasing community-driven research.
+[08/05/2026 - 1w] A volunteer mentor supporting students in Hong Kong through the I2N program, highlighting partnerships between businesses and educational institutions.
+[07/05/2026 - 1w] An open day event bringing together leaders and innovators from the Upper Hunter region to discuss future planning and investment opportunities.
+[03/05/2026 - 2w] The successful completion of the first TEDx salon in Newcastle, inspiring community engagement and discussion.
+[29/04/2026 - 2w] A local volunteer group raises significant funds for cancer research; a contribution towards advancements in medical research.
+[23/04/2026 - 3w] A visit from NHMRC representatives to discuss culturally safe healthcare practices, emphasizing community involvement in healthcare.
+[23/04/2026 - 3w] Launch of a blueprint for FEE-FREE University Ready programs, showcasing the university's commitment to enhancing educational access.
+[22/04/2026 - 3w] Official opening of a building on Mann St in Gosford, signifying business expansion and community development.</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/university-of-newcastle/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="16" t="inlineStr">
+        <is>
+          <t>Dr Eva Low</t>
+        </is>
+      </c>
+      <c r="B87" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C87" s="17" t="inlineStr">
+        <is>
+          <t>Dr Eva Low joins Sydney Health Executive Education’s public profile as a highly experienced orthodontist (--/--/----)
+A public profile highlights Dr Eva Low as a highly experienced orthodontist with over 20 years of practice, indicating established professional growth and recognition within the Sydney health education network.
+Liverpool Orthodontics profiles Dr Eva Low as a specialist orthodontist serving Liverpool NSW (--/--/----)
+Liverpool Orthodontics features Dr Eva Low on its site, noting her long-standing practice and specialist orthodontic expertise, which suggests continued practice growth and established presence in the local market.
+Orthodontics Australia lists Liverpool Orthodontics practice with Dr Eva Low (--/--/----)
+The Orthodontics Australia practice directory includes Liverpool Orthodontics and notes Dr Eva Low’s years of practice and University of Sydney training, supporting visibility and credibility for the Liverpool-based clinic.</t>
+        </is>
+      </c>
+      <c r="D87" s="17" t="inlineStr"/>
+      <c r="E87" s="16" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="16" t="inlineStr">
+        <is>
+          <t>EC Group Pty Ltd (Unit 10, 24 Vore Street, Silverwater NSW 2128, Australia)</t>
+        </is>
+      </c>
+      <c r="B88" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C88" s="17" t="inlineStr">
+        <is>
+          <t>Apprenticeship and Undergraduate Hiring Underscore EC Group’s Growth in Sydney (01/06/2024)
+EC Group, headquartered in Silverwater, NSW, has highlighted the expansion of its apprenticeship programs and undergraduate engineer positions as a central driver of the company’s growth. In its updated ‘About Us’ materials, the firm notes that structured early‑career recruitment, combined with a focus on diversity and ongoing training, has supported its rise to being recognised nationally as a market leader in building automation innovation, energy management and technical support across the commercial, health, hotel, retail, education and industrial sectors. While no specific intake numbers are disclosed, the emphasis on growing engineering talent signals continuing workforce expansion and demand for its services.</t>
+        </is>
+      </c>
+      <c r="D88" s="17" t="inlineStr"/>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/ec-group-ecgroup/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="16" t="inlineStr">
+        <is>
+          <t>ELPRO Technologies</t>
+        </is>
+      </c>
+      <c r="B89" s="16" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="C89" s="17" t="inlineStr">
+        <is>
+          <t>Aquamonix acquires ELPRO Technologies from Eaton (01/08/2021)
+Aquamonix announced its acquisition of ELPRO Technologies, indicating ELPRO’s 35-year legacy would continue and that its products and services would remain globally available. The announcement suggests business continuity and growth through ownership change and continued market reach.</t>
+        </is>
+      </c>
+      <c r="D89" s="17" t="inlineStr">
+        <is>
+          <t>[17/05/2026 - 2d] Attended ISHM Conference to showcase ELPRO Quantum Ecosystem with substantial interest from industry leaders, highlighting collaboration opportunities.
+[10/05/2026 - 1w] Discussed the evolution of industrial wireless systems, promoting the ELPRO Quantum Ecosystem as a key technology for future industrial automation.
+[24/04/2026 - 3w] Showcased innovations and strengthened partnerships at major industry events, indicating a strong market interest and alignment to industry needs.
+[20/04/2026 - 4w] Returned from a successful trip to the USA with positive market feedback on the Quantum Ecosystem, emphasizing global expansion and partner engagement.</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/elprotechnologies/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="inlineStr">
+        <is>
+          <t>ESP (Auckland, New Zealand)</t>
+        </is>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>Auckland</t>
+        </is>
+      </c>
+      <c r="C90" s="17" t="inlineStr"/>
+      <c r="D90" s="17" t="inlineStr"/>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/data-doctors-nz-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>Eden Orthodontics</t>
+        </is>
+      </c>
+      <c r="B91" s="16" t="inlineStr">
+        <is>
+          <t>Auckland</t>
+        </is>
+      </c>
+      <c r="C91" s="17" t="inlineStr"/>
+      <c r="D91" s="17" t="inlineStr"/>
+      <c r="E91" s="16" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="inlineStr">
+        <is>
+          <t>Electrical Engineering Equipment</t>
+        </is>
+      </c>
+      <c r="B92" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C92" s="17" t="inlineStr"/>
+      <c r="D92" s="17" t="inlineStr"/>
+      <c r="E92" s="16" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="16" t="inlineStr">
+        <is>
+          <t>Electronic Component Distributor (Australia)</t>
+        </is>
+      </c>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C93" s="17" t="inlineStr"/>
+      <c r="D93" s="17" t="inlineStr"/>
+      <c r="E93" s="16" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="16" t="inlineStr">
+        <is>
+          <t>Elisa Systems Pty Ltd (21 Smallwood St, Underwood QLD 4119, Australia)</t>
+        </is>
+      </c>
+      <c r="B94" s="16" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="C94" s="17" t="inlineStr">
+        <is>
+          <t>NEW AND IMPROVED SESAME KIT (15/03/2024)
+Elisa Systems announced an upgraded sesame allergen ELISA kit with improved sensitivity and performance for food manufacturers and laboratories. The new version enhances detection limits and robustness, strengthening the company’s product portfolio in allergen diagnostics and supporting growth in its core testing markets.
+New Elisa Systems Total Milk Kit (10/11/2023)
+Elisa Systems released a new Total Milk ELISA kit designed to detect milk proteins in a wide range of food matrices. The product expands the company’s allergen testing range and positions it to capture more demand from manufacturers needing comprehensive dairy allergen monitoring, indicating ongoing product-line expansion.
+Elisa Systems test kits helping to solve an international puzzle (05/06/2023)
+Elisa Systems highlighted that its allergen test kits were used by investigators in an international food safety case, demonstrating the reach and real‑world impact of its technology. The exposure reinforces the company’s global credibility and supports growth through increased recognition and potential new international customers.
+New sensitive peanut kit (20/02/2022)
+Elisa Systems introduced a highly sensitive peanut allergen ELISA kit aimed at detecting very low levels of peanut contamination in foods. This launch broadens its allergen testing portfolio, improves its competitive positioning in global diagnostics, and supports revenue growth by meeting rising regulatory and customer sensitivity requirements.</t>
+        </is>
+      </c>
+      <c r="D94" s="17" t="inlineStr"/>
+      <c r="E94" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/elisa-systems-pty-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="inlineStr">
+        <is>
+          <t>EllisCo (Auckland, NZ – leisure, travel &amp; tourism)</t>
+        </is>
+      </c>
+      <c r="B95" s="16" t="inlineStr">
+        <is>
+          <t>Auckland</t>
+        </is>
+      </c>
+      <c r="C95" s="17" t="inlineStr"/>
+      <c r="D95" s="17" t="inlineStr"/>
+      <c r="E95" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/data-doctors-nz-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="16" t="inlineStr">
+        <is>
+          <t>Elumina eLearning</t>
+        </is>
+      </c>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C96" s="17" t="inlineStr">
+        <is>
+          <t>Elumina highlights rapid company growth and investment in people on revamped careers page (01/03/2024)
+On its careers page, Elumina eLearning emphasises "rapid growth" driven by continuous learning and notes increased investment in staff development and new opportunities. The messaging reflects ongoing expansion and an active hiring posture as the company scales its operations in digital assessments and online learning.
+Elumina eLearning targets 50 million global learners with scalable digital assessment platform (23/02/2024)
+Elumina eLearning, an Australian-owned edtech company headquartered in Sydney, has articulated an ambitious growth mission to power education outcomes for 50 million learners globally by 2025. The company highlights rapid expansion of its digital assessment solutions for universities, medical colleges, professional associations and government bodies, underscoring strong demand for scalable, customisable online assessment software.
+Elumina eLearning scales high-stakes assessment delivery to over 500,000 exams per year (23/02/2024)
+According to its Australian EdTech Directory profile, Elumina eLearning now delivers more than 500,000 high‑stakes assessments annually for global educational institutions, medical colleges, universities, professional associations and government agencies. This volume milestone reflects substantial platform adoption and operational scale in the digital assessment market.
+Elumina eLearning grows to 100+ staff supporting global assessment clients (23/02/2024)
+Elumina eLearning reports a team of more than 100 employees supporting its digital assessment, online learning and enterprise solutions. The headcount figure, noted in its Australian EdTech Directory listing, indicates sustained hiring and organisational growth to meet increasing demand from education and government clients.
+Elumina launches AI-powered Assess App to streamline digital assessment lifecycle (15/01/2024)
+Elumina eLearning has introduced its AI-powered Assess App, positioned as a way for institutions and organisations to manage the entire assessment process—including development, delivery and marking—within a single platform. The product launch signals continued product innovation and an expansion of Elumina’s capabilities in automating and scaling assessments.</t>
+        </is>
+      </c>
+      <c r="D96" s="17" t="inlineStr"/>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/eluminaelearning/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="16" t="inlineStr">
+        <is>
+          <t>Embrace Orthodontists (Canberra, ACT, Australia)</t>
+        </is>
+      </c>
+      <c r="B97" s="16" t="inlineStr">
+        <is>
+          <t>Canberra</t>
+        </is>
+      </c>
+      <c r="C97" s="17" t="inlineStr">
+        <is>
+          <t>Embrace Orthodontists recognised among Canberra’s best orthodontic practices (15/04/2025)
+Local Canberra lifestyle outlets Region Media and Canberra Daily both named Embrace Orthodontists as one of the best orthodontic practices in Canberra, highlighting its award‑winning status, leading role in Invisalign and braces treatments, and strong patient experience. This recognition reinforces the practice’s market position and brand strength in the Canberra region.
+Embrace Orthodontists expands to three practices across Canberra (10/03/2024)
+Embrace Orthodontists has grown its physical footprint to three clinics in Canberra—Belconnen, Manuka and Gungahlin—providing increased access to specialist orthodontic care across North and South Canberra and the Gungahlin growth corridor. The expansion reflects sustained demand for orthodontic and Invisalign services and indicates operational growth beyond its original base in Manuka.
+Embrace Orthodontists promoted as a leading Invisalign provider in Canberra (01/09/2023)
+Embrace Orthodontists is promoted on its corporate site as Canberra’s leading Invisalign provider and a Black Diamond Invisalign Provider, a designation typically awarded to practices with high case volumes. This status suggests strong patient throughput, deep clinical experience with clear aligner therapy, and a solid revenue base from Invisalign-related services.
+Embrace Orthodontists scales operations with multi‑site service model (20/02/2023)
+Through its Manuka headquarters and additional Belconnen and Gungahlin practices, Embrace Orthodontists has implemented a multi‑site service model with extended weekday opening hours. This structure supports higher patient capacity, improved accessibility for different regions of Canberra, and operational scalability for the allied health business.</t>
+        </is>
+      </c>
+      <c r="D97" s="17" t="inlineStr"/>
+      <c r="E97" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/embrace-orthodontists/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="16" t="inlineStr">
+        <is>
+          <t>Emergent Group</t>
+        </is>
+      </c>
+      <c r="B98" s="16" t="inlineStr">
+        <is>
+          <t>New South Wales</t>
+        </is>
+      </c>
+      <c r="C98" s="17" t="inlineStr">
+        <is>
+          <t>Emergent Group Leans Into The Future (01/01/2024)
+Emergent Group completed a three-month recruitment campaign called The Network Effect, signaling a push to evolve the business and strengthen its workforce. The article highlights the company’s strategy to leverage network theory and adapt for future growth.
+Emergent Group launches campaign to attract workforce talent (01/06/2023)
+Emergent Group launched The Network Effect recruitment campaign to attract talent across engineering, science, and leadership roles. The initiative included referral rewards, aimed to fill vacancies, and explicitly encouraged nominations of women candidates to help address gender imbalance in the team.</t>
+        </is>
+      </c>
+      <c r="D98" s="17" t="inlineStr">
+        <is>
+          <t>[20/04/2026 - 4w] Highlighting the significant work of the product development team at Novecom, focusing on their new 'SureWaste' technology that addresses waste in the health sector.</t>
+        </is>
+      </c>
+      <c r="E98" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/emergentgroup/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="inlineStr">
+        <is>
+          <t>EncompaaS</t>
+        </is>
+      </c>
+      <c r="B99" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C99" s="17" t="inlineStr">
+        <is>
+          <t>Atturra expands AI offerings through partnership with EncompaaS (11/11/2025)
+Technology services provider Atturra entered a strategic partnership with EncompaaS to expand its artificial intelligence offerings and support successful enterprise adoption of agentic AI. Under the partnership, Atturra will combine its consulting and delivery expertise with EncompaaS’s intelligent data-preparation and information management platform, helping clients build AI-ready, governed data foundations across sectors such as defence, government, education and manufacturing.
+Atturra and EncompaaS partner to ensure successful agentic AI adoption by enterprises (11/11/2025)
+Atturra and EncompaaS jointly announced an Australia-based strategic partnership focused on enabling enterprises to re-engineer business processes and confidently adopt agentic AI. The collaboration leverages EncompaaS’s AI-powered platform for data discovery, classification and governance along with Atturra’s technology deployment capabilities, positioning EncompaaS more deeply within large enterprise and regulated industries pursuing advanced AI initiatives.
+EncompaaS named finalist in InnovationAus 2024 Awards for Excellence (10/09/2024)
+NSW-based EncompaaS was named a finalist in the InnovationAus 2024 Awards for Excellence, recognising its AI-powered information management platform that discovers, enriches and organises structured and unstructured enterprise data. The recognition validates the company’s strategy of using AI and machine learning, including integrations with Microsoft Azure OpenAI and other AI services, to help organisations extract value from data sprawl while maintaining compliance and security.
+EncompaaS launches focused ‘Get AI Ready’ data-preparation offering (15/04/2024)
+EncompaaS introduced a refined market proposition under the banner “Get AI Ready with Beautifully Prepared Data,” emphasising automated preparation of unstructured data for AI use. The offering underscores the company’s growth strategy around AI data readiness, enabling enterprises to normalise and govern content across repositories and make it suitable for advanced AI services, reinforcing EncompaaS’s positioning in the emerging AI infrastructure and data-preparation space.
+EncompaaS positions platform as foundation for AI-ready enterprise data (01/03/2024)
+Through updates highlighted on its corporate site, EncompaaS is positioning its intelligent information management platform as a way for regulated enterprises to transform fragmented, high-risk content into a secure, AI-ready foundation. The Sydney-based company emphasises new AI-powered capabilities for discovering and organising structured and unstructured data across cloud, on‑premises and hybrid environments, supporting enterprise adoption of tools such as Microsoft Copilot and Azure OpenAI while maintaining compliance and governance.
+NSW Department of Planning and Environment adopts EncompaaS cloud platform (16/08/2022)
+The NSW Department of Planning and Environment implemented the EncompaaS cloud platform to improve compliance and records management in its Microsoft 365 environment. This government deployment follows Bendigo and Adelaide Bank’s selection of EncompaaS to automate electronic document compliance, highlighting growing traction for the company’s cloud-based governance and compliance solution in both public sector and financial services.
+EncompaaS in $14m capital raise, targets global growth (08/10/2021)
+Enterprise compliance SaaS provider EncompaaS completed a AU$14 million capital raise led by CVC Emerging Companies, Future Now Capital and Marshall Investments to accelerate its scale‑up strategy. The funding is earmarked to expand international sales, further develop its cloud-based information governance platform, and support global market entry. The company has recently secured major contracts with one of Australia’s top five banks and a large NSW government department, and has established offices in the UK and US, adding a major European bank to its client list.</t>
+        </is>
+      </c>
+      <c r="D99" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Collaboration with Serena Williams and Reckitt to support underrepresented founders.
+[27/04/2026 - 3w] LinkedIn's recognition as the most-cited domain for professional inquiries, showcasing success.
+[22/04/2026 - 3w] Announcement of new executive appointments at LinkedIn indicating leadership growth.</t>
+        </is>
+      </c>
+      <c r="E99" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="16" t="inlineStr">
+        <is>
+          <t>Endotherapeutics (Sydney, Australia)</t>
+        </is>
+      </c>
+      <c r="B100" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C100" s="17" t="inlineStr">
+        <is>
+          <t>Endotherapeutics Awarded EcoVadis Bronze Medal for Sustainability (18/09/2025)
+Endotherapeutics, the Sydney-based medical technology distributor, was awarded a Bronze Medal by EcoVadis for its sustainability performance. The recognition reflects the company’s progress in areas such as environmental practices, ethics, and responsible procurement, and positions Endotherapeutics more competitively with hospitals and health systems that increasingly factor ESG credentials into supplier selection. The medal supports the company’s brand reputation and can help underpin future commercial growth and partnership opportunities.</t>
+        </is>
+      </c>
+      <c r="D100" s="17" t="inlineStr">
+        <is>
+          <t>[12/05/2026 - 1w] Announcement of exclusive partnership with Bien-Air Surgery for distribution of power tools in Australia.
+[11/05/2026 - 1w] Celebration of International Nurses Day while encouraging hiring and career exploration.
+[23/04/2026 - 3w] Announcement of exclusive partnership as the sole distributor for VARIXIO in Australia and New Zealand.</t>
+        </is>
+      </c>
+      <c r="E100" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/endotherapeutics/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>Energetica (152 Elizabeth St, Melbourne, VIC 3000, Australia)</t>
+        </is>
+      </c>
+      <c r="B101" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C101" s="17" t="inlineStr">
+        <is>
+          <t>No verified growth-related news articles found for Energetica at 152 Elizabeth St, Melbourne (01/01/1900)
+A search of public web sources and industry news (renewable energy in Victoria and Australia more broadly) did not return any verifiable news articles specifically about Energetica headquartered at 152 Elizabeth St, Melbourne, VIC 3000, Australia. Available search results referenced other entities in the renewable energy sector (such as government initiatives, large battery projects, and other developers) but none could be confidently matched to this exact company and address. To avoid mixing it up with similarly named firms, no unverified or ambiguous items are included.</t>
+        </is>
+      </c>
+      <c r="D101" s="17" t="inlineStr"/>
+      <c r="E101" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/energetica.io/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="16" t="inlineStr">
+        <is>
+          <t>Energy-Tec (Perth, Western Australia)</t>
+        </is>
+      </c>
+      <c r="B102" s="16" t="inlineStr">
+        <is>
+          <t>Perth</t>
+        </is>
+      </c>
+      <c r="C102" s="17" t="inlineStr">
+        <is>
+          <t>Energy-Tec expands advanced metering and solar portfolio across WA and eastern states (01/03/2023)
+Perth-based Energy-Tec has broadened its operations from traditional sub‑meter reading and billing into a full technical division delivering Advanced Metering Infrastructure (AMI) and large‑scale solar solutions. The company reports having implemented AMI projects with large solar systems at more than 20 commercial properties across Western Australia and on the eastern seaboard, and now services thousands of properties nationwide. This marks a significant expansion of its renewable and smart‑metering footprint in retail, commercial, industrial, strata, retirement living, airport estates, educational campuses and government buildings.
+Long‑term partnership with Perth Airport underpins Energy-Tec’s growth in embedded network metering (01/06/2022)
+EnergyTec (Energy-Tec) has been a key metering and energy‑management partner to Perth Airport for more than five years, supporting the airport’s transition to advanced and smart meter technology across its 22 kV embedded distribution network. The ongoing role in the Perth Airport Metering Transformation Project highlights the company’s growth in complex embedded‑network projects and reinforces its position as a specialist provider of metering solution management for large infrastructure clients.
+Energy-Tec scales sustainability and renewable solutions offering for commercial property sector (01/09/2021)
+Energy-Tec has expanded its core services beyond sub‑metering into integrated sustainability consulting and renewable energy solutions for commercial property owners. By offering customised ‘energy roadmaps’ designed to prepare assets for the next decade of energy‑market evolution, the company has increased its service scope to include end‑to‑end metering, energy efficiency and renewable project delivery across thousands of properties in Perth, regional Western Australia and nationally.</t>
+        </is>
+      </c>
+      <c r="D102" s="17" t="inlineStr">
+        <is>
+          <t>[14/05/2026 - 5d] EnergyTec supports the 2026 Property Council WA Awards and commends nominees, indicating company recognition.
+[28/04/2026 - 3w] Our client-facing team is a finalist for Property Council WA Team of the Year, showcasing team excellence.
+[21/04/2026 - 4w] EnergyTec is recognized as a finalist in the SCA Australasia Awards, demonstrating industry acknowledgment and growth.</t>
+        </is>
+      </c>
+      <c r="E102" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/energytecholdings/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="inlineStr">
+        <is>
+          <t>Engineering Supplies</t>
+        </is>
+      </c>
+      <c r="B103" s="16" t="inlineStr">
+        <is>
+          <t>Perth</t>
+        </is>
+      </c>
+      <c r="C103" s="17" t="inlineStr">
+        <is>
+          <t>Engineering Supplies: Online Electrical Supply Store In Welshpool (01/01/2025)
+This company profile highlights Engineering Supplies’ long-standing presence in the Australian electrical market, its broad product range, and its role as a distributor for multiple major brands. While not a traditional news article, it indicates business scale and ongoing market activity rather than a specific growth event.
+Engineering Supplies drawing exceptional interest within the Retail industry (01/01/2025)
+This company overview notes that Engineering Supplies is attracting exceptional interest within its industry, which can be interpreted as a sign of strong market momentum. It suggests increased attention around the business, though the page does not provide a specific growth announcement.</t>
+        </is>
+      </c>
+      <c r="D103" s="17" t="inlineStr"/>
+      <c r="E103" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/engineering-supplies-au/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="inlineStr">
+        <is>
+          <t>EpiSoft</t>
+        </is>
+      </c>
+      <c r="B104" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C104" s="17" t="inlineStr">
+        <is>
+          <t>EpiSoft launches My Health Record upload capability for oncology treatment summaries (01/01/2024)
+EpiSoft announced an Australian-first innovation enabling treatment event summaries covering a full cycle of care to be seamlessly uploaded to My Health Record through its medical oncology management platform, indicating continued product expansion and platform advancement.
+The San partners with EpiSoft for integrated cancer centre (01/01/2019)
+Sydney Adventist Hospital selected EpiSoft’s Cancer CareZone cloud-based clinical information system for its new Integrated Cancer Centre, reflecting a major partnership and deployment in a large hospital redevelopment.
+EpiSoft secures Federal Government grant and private investment to accelerate global expansion (01/01/2014)
+EpiSoft’s co-founders said the company received a $250,000 Federal Government grant and later attracted $1 million in private investment, which was expected to accelerate global expansion of its cloud-based healthcare software platform.</t>
+        </is>
+      </c>
+      <c r="D104" s="17" t="inlineStr"/>
+      <c r="E104" s="16" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
+        <is>
+          <t>Evado (Melbourne, Australia)</t>
+        </is>
+      </c>
+      <c r="B105" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C105" s="17" t="inlineStr"/>
+      <c r="D105" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Collaboration with Serena Williams and Reckitt to enhance business networks.
+[24/04/2026 - 3w] Celebration of Fernando Mendoza's appointment.
+[22/04/2026 - 3w] Congratulatory post on new CEO and President appointments, indicating positive leadership changes.</t>
+        </is>
+      </c>
+      <c r="E105" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="inlineStr">
+        <is>
+          <t>Everlink (10 Cypress St, Tauranga, Bay of Plenty, 3110, New Zealand)</t>
+        </is>
+      </c>
+      <c r="B106" s="16" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C106" s="17" t="inlineStr">
+        <is>
+          <t>Everlink invests in integrated hardware–software platform for fuel‑chain visibility (05/11/2019)
+Everlink has enhanced its core offering by investing in an integrated hardware–software platform designed to ‘connect every link in the fuel supply chain’. The platform provides real‑time visibility and control over fuel usage and inventory, aimed at improving efficiency and compliance for industrial customers. This represents a strategic product‑development initiative that deepens its capabilities in electronic monitoring and control systems manufactured from its Tauranga base.
+Everlink strengthens reputation as a global fuel‑management solutions provider (20/07/2018)
+Everlink, headquartered in Tauranga, has continued to build an international customer base for its purpose‑built hardware and software that manage, monitor, and maintain fuel flows across complex supply chains. The company reports a proven track record of success around the world and positions itself as a trusted name in fuel management, highlighting sustained export growth and increasing adoption of its electronic fuel‑management systems in overseas markets.
+Everlink broadens product range into automated fluid management for heavy industry (10/09/2015)
+Building on its origins as a New Zealand fuel‑management specialist, Everlink has grown its offering to encompass a wider suite of automated fluid management and control products tailored for heavy industries such as rail, civil engineering, mining, and transport. This diversification reflects product‑line expansion from traditional fuel management into broader electronic control and monitoring solutions for industrial fluids, leveraging its in‑house design and manufacturing capabilities in Tauranga.
+Everlink expands Australian presence with dedicated Everlink Australia entity (15/03/2015)
+Everlink, founded in Tauranga in 2001, has expanded its reach by establishing a dedicated Australian operation (Everlink Australia) to design and manufacture fuel and fluid management products for sectors including rail, civil engineering, mining, and transport. The move formalised and scaled up its export activities from New Zealand into Australia, signalling geographic expansion and increased manufacturing capacity beyond its Tauranga base.</t>
+        </is>
+      </c>
+      <c r="D106" s="17" t="inlineStr">
+        <is>
+          <t>[10/05/2026 - 1w] Announces a partnership with Mansfield Group to enhance diesel filtration systems at client sites.
+[28/04/2026 - 3w] Acknowledges the distributor's efforts in Papua New Guinea, hinting at market expansion.
+[27/04/2026 - 3w] Mentions a shift towards integrated dispensing solutions as a sign of market adaptation.
+[19/04/2026 - 1mo] Describes the company's participation in an expo and connection with clients through partnerships.</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/everlink-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="inlineStr">
+        <is>
+          <t>Exergenics</t>
+        </is>
+      </c>
+      <c r="B107" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C107" s="17" t="inlineStr">
+        <is>
+          <t>Exergenics secures Accelerating Commercialisation Grant for 2023/2024 financial year (01/07/2023)
+Exergenics announced it had been awarded an Accelerating Commercialisation Grant for 2023/2024 to support development and scaling of its AI-powered cloud-based chiller plant optimisation platform. The funding was positioned as a boost for product development and market expansion, with claims of enabling up to 35% energy savings.
+How Exergenics' machine learning can help make air conditioning more energy efficient (01/06/2021)
+University of Melbourne coverage highlighted Exergenics as a Melbourne startup using machine learning to optimise large-scale commercial air conditioning and refrigeration systems. The article noted that Exergenics was deploying pilots across multiple sites, had achieved energy savings of 5–15% in most buildings, and was raising capital to accelerate growth and expand internationally.
+Exergenics announced as winner of Start-up Proptech of the Year (01/05/2021)
+Exergenics was recognised with the 'Start-up Proptech of the Year' award from the Proptech Association of Australia, signalling external industry validation and momentum for the Melbourne-based company.</t>
+        </is>
+      </c>
+      <c r="D107" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Announcement of partnership with Serena Williams and Reckitt to promote networking.
+[27/04/2026 - 3w] LinkedIn recognized as the #1 cited domain for professional queries on AI search engines.
+[22/04/2026 - 3w] Announcement of new CEO and President roles within LinkedIn.</t>
+        </is>
+      </c>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="16" t="inlineStr">
+        <is>
+          <t>Expressway Spares Pty Ltd</t>
+        </is>
+      </c>
+      <c r="B108" s="16" t="inlineStr">
+        <is>
+          <t>New South Wales</t>
+        </is>
+      </c>
+      <c r="C108" s="17" t="inlineStr">
+        <is>
+          <t>Expressway Spares celebrates 60 years of growth, legacy and strategy (15/04/2024)
+In a feature article, Expressway Spares marked its 60th year in business, outlining sustained growth from a small wrecking yard to a major supplier of new, used and reconditioned parts for Caterpillar and Hitachi equipment. The piece highlighted expansion to multiple branches across three states, the scaling of its workforce to more than 380 employees, significant investment in workshops and component rebuild facilities, and a long‑term strategy focused on customer service and international sourcing of machinery and parts.
+Expressway Spares named 2022 Workplace Safety Champions by SafeWork NSW (15/11/2022)
+Expressway Spares was recognised as the 2022 Workplace Safety Champions at the SafeWork NSW Excellence Awards. The award highlighted the company’s strong safety culture, systems and initiatives across its workshops and sites, reinforcing its position as a leading and responsible employer within the heavy equipment parts and machinery sector.
+Expressway Spares grows into one of Australia’s largest independent heavy equipment parts suppliers (01/08/2021)
+A NAB Business profile described how Expressway Spares evolved into a sophisticated aftermarket parts enterprise supplying the mining, construction and logging sectors. The article noted its expansion to five offices across three states, a large headcount at its New South Wales head office, and its position as one of the largest private independent dealers of parts and components suitable for Caterpillar internationally. The company’s model of acquiring, stripping and reconditioning heavy machinery from around the world was highlighted as a key driver of ongoing growth and export activity.
+Perth branch opens as Expressway Spares expands national footprint (01/02/2020)
+Expressway Spares reported the opening of its Perth branch in Western Australia, extending its service coverage to more mining and earthmoving customers across the state. The new location added local inventory, workshop capability and customer support, strengthening the company’s presence in key resource regions and supporting ongoing expansion beyond its New South Wales base.
+Expressway Spares adds AS/NZS 4801 and ISO 14001 certifications to scope (01/06/2019)
+Expressway Spares announced that it had expanded the scope of its management systems to include AS/NZS 4801 (occupational health and safety) and ISO 14001 (environmental management). Achieving these additional certifications formalised the company’s commitment to safety and environmental performance across its operations and supported growth with larger mining and construction customers that require certified suppliers.</t>
+        </is>
+      </c>
+      <c r="D108" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] The company is opening applications for apprenticeships, indicating growth through recruitment and team expansion.</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/expressway-spares-pty-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="16" t="inlineStr">
+        <is>
+          <t>Ezihealth</t>
+        </is>
+      </c>
+      <c r="B109" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C109" s="17" t="inlineStr"/>
+      <c r="D109" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Partnership announcement with Serena Williams and Reckitt to leverage networks for small businesses.
+[27/04/2026 - 3w] Highlighting LinkedIn's dominance as the most-cited domain for AI queries indicates market expansion and relevance.
+[22/04/2026 - 3w] Announcement of new leadership roles at LinkedIn, indicating company leadership changes.</t>
+        </is>
+      </c>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="16" t="inlineStr">
+        <is>
+          <t>FRAMECAD</t>
+        </is>
+      </c>
+      <c r="B110" s="16" t="inlineStr">
+        <is>
+          <t>Auckland</t>
+        </is>
+      </c>
+      <c r="C110" s="17" t="inlineStr">
+        <is>
+          <t>FRAMECAD launches ‘Steel Framing Connections’ podcast to showcase global CFS project growth (15/04/2026)
+FRAMECAD has launched a new monthly podcast series, ‘Steel Framing Connections’, focused on real-world applications of cold-formed steel (CFS) framing in global construction markets. Produced from Auckland, the series features industry leaders and project case studies highlighting how steel framing is improving speed, efficiency and performance across residential, commercial and modular construction. The initiative supports FRAMECAD’s market development and brand-building strategy as it promotes its steel framing systems and software to a broader international audience.
+FRAMECAD appoints Aaron Wright as CEO to lead next phase of global growth (02/03/2026)
+FRAMECAD, the Auckland-based steel frame construction technology company, has appointed Aaron Wright as CEO as it enters its next phase of global growth. Wright steps up from his role as Chief Operations Officer, which he has held since April 2024. Founder and long-time CEO Mark Taylor becomes Executive Director of the FRAMECAD Group. The leadership change is positioned as a move to accelerate international expansion of FRAMECAD’s end-to-end cold-formed steel (CFS) construction system, roll-forming technology, and digital design solutions for residential and commercial projects worldwide.
+FRAMECAD launches FRAMECAD Nexa, expanding its steel frame building technology suite (22/10/2024)
+FRAMECAD announced the launch of FRAMECAD Nexa, described as a significant enhancement to its steel frame building innovation platform. As an advanced end-to-end design and build system provider, FRAMECAD is extending its product and software offering to enable faster, more efficient cold-formed steel construction. The launch underscores the company’s ongoing investment in product development to support businesses, governments and communities with rapid, durable, cost-effective buildings worldwide.
+FRAMECAD moves into new Glen Innes premises and begins new R&amp;D contracts (03/11/2011)
+New Zealand Government communications highlighted that steel-frame export company FRAMECAD has relocated into new premises in Glen Innes, Auckland, as it commences work on several new research and development contracts. The move into larger facilities and the securing of multiple R&amp;D projects signal expansion of FRAMECAD’s innovation capability and export-focused operations in cold-formed steel construction technology.</t>
+        </is>
+      </c>
+      <c r="D110" s="17" t="inlineStr">
+        <is>
+          <t>[10/05/2026 - 1w] Announcement of Aaron Wright as new CEO to lead growth efforts.
+[08/05/2026 - 1w] Example of how light steel frame technology helped rebuild homes after floods in Brazil.
+[29/04/2026 - 2w] Case study on the rapid adoption of steel framing in a townhouse project.
+[28/04/2026 - 3w] Launch of the Steel Framing Connections podcast focusing on industry insights.
+[28/04/2026 - 3w] Grupo SteelCorp's initiative to rebuild communities with light steel frame homes.</t>
+        </is>
+      </c>
+      <c r="E110" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/framecad-limited/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
+        <is>
+          <t>FYI (FYI Software Pty Ltd), Adelaide, South Australia</t>
+        </is>
+      </c>
+      <c r="B111" s="16" t="inlineStr">
+        <is>
+          <t>Adelaide</t>
+        </is>
+      </c>
+      <c r="C111" s="17" t="inlineStr">
+        <is>
+          <t>FYI emerges as Australia and New Zealand’s fastest‑growing automated document and practice management platform (05/03/2024)
+Trade coverage in outlets such as Accountants Daily and Accounting Times describes FYI as Australia and New Zealand’s fastest‑growing automated document and practice management software, now transforming how more than 30,000 accountants operate. The articles highlight rapid user adoption across accounting firms and emphasise FYI’s automation features, positioning the Adelaide‑headquartered company as a high‑growth player in the accounting technology market.
+FYI scales operations across Australia, New Zealand and the UK from its Adelaide headquarters (15/09/2023)
+In updated company information, FYI reports that it is headquartered in Adelaide’s East End and now has a growing, distributed team across Australia, New Zealand and the United Kingdom. This geographic expansion of staff and operations signals sustained growth in demand for FYI’s cloud‑based document and practice management platform within multiple regions.</t>
+        </is>
+      </c>
+      <c r="D111" s="17" t="inlineStr"/>
+      <c r="E111" s="16" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="16" t="inlineStr">
+        <is>
+          <t>Factory Controls Pty Ltd (65 Douro Street, North Geelong, VIC 3215, Australia)</t>
+        </is>
+      </c>
+      <c r="B112" s="16" t="inlineStr">
+        <is>
+          <t>Victoria</t>
+        </is>
+      </c>
+      <c r="C112" s="17" t="inlineStr">
+        <is>
+          <t>Factory Controls strengthens automation offering through new technology partnerships (01/03/2024)
+Factory Controls, a Victorian-based industrial automation and controls specialist headquartered in North Geelong, has expanded its partner network with a series of new and upgraded agreements with leading global vendors in PLCs, drives, industrial networking and safety systems. The company highlighted that its strategic partnerships are aimed at delivering more integrated automation solutions for local manufacturers and infrastructure projects, reinforcing its role in Victoria’s advanced manufacturing and process control supply chains. While financial details were not disclosed, the broadened partner portfolio indicates a growth focus on higher‑value engineering, systems integration and long‑term service contracts.</t>
+        </is>
+      </c>
+      <c r="D112" s="17" t="inlineStr"/>
+      <c r="E112" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/factory-controls/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="16" t="inlineStr">
+        <is>
+          <t>FeeSynergy</t>
+        </is>
+      </c>
+      <c r="B113" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C113" s="17" t="inlineStr">
+        <is>
+          <t>FeeSynergy partners with Equifax to integrate business credit scoring for accounting and legal firms (22/05/2023)
+Melbourne-based debtor management fintech FeeSynergy announced a strategic partnership with global data and analytics company Equifax to enhance how accounting and legal firms assess client credit risk. The integration allows FeeSynergy users to access Equifax business credit scores and credit reports directly within their risk assessment workflows, providing greater visibility of clients’ creditworthiness and ability to pay. FeeSynergy’s managing director Malcolm Ebb described the collaboration as ‘ground-breaking’ and noted that the product had been in development for over two years, positioning the company to deliver deeper risk insights and identify new business advisory opportunities for its professional-services customer base.
+FeeSynergy strengthens market position as leading AR automation platform for accounting and legal firms in ANZ (15/03/2022)
+FeeSynergy highlighted continued growth as the leading accounts receivable automation platform tailored to accounting and legal firms across Australia and New Zealand. The company reports widespread adoption of its FeeSynergy Collect platform and Payment Gateway, with client testimonials citing outcomes such as reducing debtor days by around two-thirds within six months of implementation and shifting the majority of client payments to automated channels. This traction underscores FeeSynergy’s expanding customer base and recurring SaaS revenue footprint in the professional-services sector.</t>
+        </is>
+      </c>
+      <c r="D113" s="17" t="inlineStr"/>
+      <c r="E113" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/feesynergy-finance-p-l/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="16" t="inlineStr">
+        <is>
+          <t>FilePro</t>
+        </is>
+      </c>
+      <c r="B114" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C114" s="17" t="inlineStr">
+        <is>
+          <t>Actionstep Acquires Australian Legal Software Company FilePro (31/08/2023)
+Cloud practice management provider Actionstep acquired Perth-based legal software business FilePro, combining two practice management platforms focused on mid-sized law firms. The deal is positioned as a growth step for FilePro’s customers, who are expected to gain access to expanded cloud technologies and increased product development investment, while strengthening Actionstep’s presence in the Australian legal software market.
+FilePro Releases Dashboard and User Interface Enhancements (23/02/2021)
+FilePro announced a set of product updates including the introduction of a new FilePro Dashboard, refreshed screen designs, and upcoming improvements to document assembly. These enhancements are part of ongoing product investment to improve usability and workflow efficiency for law firm customers across Australia.
+FilePro Board Approves Additional $1m Investment in Next-Generation Software (07/08/2017)
+FilePro’s board approved a further AU$1,000,000 investment to accelerate development of its next-generation legal practice management platform. The funding was described as a strategic move to give the company an additional competitive advantage and underpins FilePro’s product roadmap and long-term growth strategy in the legal software sector.
+FilePro Implements Five-Year National Growth Strategy (01/06/2015)
+FilePro outlined a five-year national growth strategy aimed at ensuring its longevity and continued delivery of high service and value to clients. The plan focuses on expanding its footprint with Australian law firms, enhancing its all-in-one practice management offering, and supporting ongoing product development and client support initiatives.</t>
+        </is>
+      </c>
+      <c r="D114" s="17" t="inlineStr"/>
+      <c r="E114" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/filepro/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="16" t="inlineStr">
+        <is>
+          <t>Fine Orthodontist Sydney</t>
+        </is>
+      </c>
+      <c r="B115" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C115" s="17" t="inlineStr"/>
+      <c r="D115" s="17" t="inlineStr"/>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fine-orthosydney/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="16" t="inlineStr">
+        <is>
+          <t>Flash Payments</t>
+        </is>
+      </c>
+      <c r="B116" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C116" s="17" t="inlineStr">
+        <is>
+          <t>Flash Payments announces 2024 partnership with Eastern Suburbs Rugby (15/03/2024)
+Flash Payments, the Sydney-based fintech headquartered at Level 26, 1 Bligh Street, expanded its brand reach and community presence by becoming a 2024 partner of Eastern Suburbs Rugby. The sponsorship aligns the company with a high-profile Sydney sporting organisation and is positioned as a way to showcase its innovative cross‑border and instant payment capabilities to a broader local audience while deepening ties in its home market.
+Flash Payments strengthens strategic partnership with Ripple to scale blockchain-powered cross‑border payments (10/11/2023)
+Flash Payments highlighted its role as a key Australian strategic partner of Ripple, leveraging RippleNet and On‑Demand Liquidity (ODL) to deliver faster, lower‑cost international money transfers for businesses across 40+ countries and 20+ currencies. The company emphasised scaling of its blockchain-based FX and virtual account offering, signalling operational and product expansion in global B2B and B2E payments out of its Sydney headquarters.
+Flash Payments recognised for innovation in cross‑border payment solutions (05/09/2023)
+Flash Payments reported industry recognition for its innovative cross‑border payment solutions, which use blockchain technology, competitive FX, and AI/ML‑driven fraud detection. The acknowledgment underscores the firm’s growing influence in the Australian fintech ecosystem and validates its technology-led growth strategy in secure international money transfers for businesses.
+Flash Payments joins Australian FinTech as newest member to support scaling businesses (22/08/2023)
+Australian FinTech announced Flash Payments as its newest member, spotlighting the Sydney company’s complete payment solution that spans foreign exchange, international transfers, and digital payment capabilities. Membership enhances Flash Payments’ visibility within the national fintech community and is positioned to support further business development and scaling with enterprise clients.
+Flash Payments underscores regulated status and infrastructure investment to support growth (30/06/2023)
+In an updated corporate overview, Flash Payments detailed its status as a regulated entity holding an ASIC Australian Financial Services Licence (AFSL) and AUSTRAC registration, alongside a management team with over 50 years of banking and financial services experience. The company highlighted investments in AI/ML for fraud detection, virtual accounts, and compliant infrastructure—positioning itself for continued growth in enterprise-grade international payment services from its Sydney headquarters.</t>
+        </is>
+      </c>
+      <c r="D116" s="17" t="inlineStr"/>
+      <c r="E116" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/flash-payments/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="16" t="inlineStr">
+        <is>
+          <t>Fluid Power Engineering Solutions (Sydney, Australia)</t>
+        </is>
+      </c>
+      <c r="B117" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C117" s="17" t="inlineStr">
+        <is>
+          <t>Fluid Power Engineering Solutions enters Western Australian market with Perth centre of excellence (01/11/2022)
+Fluid Power Engineering Solutions expanded beyond its East Coast base into Perth, Western Australia, establishing a local centre of excellence focused on transformers and high‑voltage assets. The new location offers a full range of turnkey solutions including smart systems and predictive maintenance, rotating equipment consultancy and maintenance, and specialist filtration services, allowing the company to tap into Western Australia’s growing industrial market and serve customers as a one‑source systems integrator.
+Fluid Power Engineering Solutions expands operations with new Wetherill Park headquarters (01/06/2020)
+Fluid Power Engineering Solutions, a privately owned hydraulic and mechanical engineering firm, relocated to a larger, more professional headquarters in Wetherill Park, Western Sydney. The move created a dedicated ‘centre of excellence’ for engineering, hydraulic and filtration solutions, and provided capacity to grow its team and service capabilities for industrial customers in the Sydney region.
+Fluid Power Engineering Solutions scales up offerings through merger of two hydraulic businesses (01/03/2018)
+The formation of Fluid Power Engineering Solutions is described as the result of a powerful combination of two successful hydraulic companies joining forces. This consolidation brought together an extensive suite of capabilities and a larger pool of specialised staff, positioning the business as a premier hydraulic service centre in a key Sydney industrial hub and enhancing its ability to deliver 360° mechanical, hydraulic and electronic solutions.</t>
+        </is>
+      </c>
+      <c r="D117" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Partnership announcement with Serena Williams and Reckitt focusing on network leverage.
+[27/04/2026 - 3w] Announcement of LinkedIn being the top-cited domain for professional queries.
+[22/04/2026 - 3w] Announcement of new leadership roles within LinkedIn indicating team growth.</t>
+        </is>
+      </c>
+      <c r="E117" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="16" t="inlineStr">
+        <is>
+          <t>FormTab Ltd (Christchurch, Canterbury Region, New Zealand)</t>
+        </is>
+      </c>
+      <c r="B118" s="16" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C118" s="17" t="inlineStr"/>
+      <c r="D118" s="17" t="inlineStr"/>
+      <c r="E118" s="16" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="16" t="inlineStr">
+        <is>
+          <t>FreightSafe (Sydney, Australia)</t>
+        </is>
+      </c>
+      <c r="B119" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C119" s="17" t="inlineStr">
+        <is>
+          <t>FreightSafe Group partners with Ofload to enhance goods protection (05/07/2024)
+Digital freight platform Ofload announced a strategic partnership with the FreightSafe Group, describing FreightSafe as a leading digital‑first freight insurance provider. The collaboration embeds FreightSafe’s technology‑driven, customised transit‑insurance solutions and high‑scale claims management into Ofload’s platform to protect customers’ goods against loss or damage. The deal underscores FreightSafe’s growth via platform integrations, expanded customer reach, and the use of advanced technology and data analytics for real‑time risk assessment.
+FreightInsure, part of FreightSafe Group, launches embedded per‑shipment cover in ANZ (15/03/2024)
+FreightInsure, the embedded insurance solution within the FreightSafe Group, detailed its offering of per‑shipment freight insurance that integrates directly into carriers’ and logistics platforms’ existing workflows. The product activates cover automatically at shipment, with FreightSafe managing claims end‑to‑end and removing liability from distributors. The service is now operating in both Australia and New Zealand, indicating regional expansion and deeper embedding of FreightSafe’s digital insurance and claims capabilities in logistics platforms.
+Lombard backs insurtech FreightInsure, part of FreightSafe Group (19/09/2023)
+Lombard Australia Holdings, parent of Assetinsure, invested capacity and support into FreightInsure, a goods‑in‑transit insurtech that sits within the FreightSafe Group. The partnership launches FreightInsure with many of FreightSafe’s largest transport and logistics clients, embedding per‑shipment insurance into carriers’ booking processes. The product offers pay‑as‑you‑go mini‑policies with cover up to $50,000 per consignment and no excess, indicating product expansion and financial backing for FreightSafe’s insurance and digital offerings in Australia (and later New Zealand).
+Insurtech Australia welcomes FreightSafe as new member (08/06/2022)
+Industry association Insurtech Australia announced that third‑party claims administrator FreightSafe has joined as a member. The move signals FreightSafe’s growing scale—managing tens of thousands of freight and marine claims annually—and its intention to engage more deeply with the Australian insurtech community. The company highlighted its proprietary claims management system, ability to finalise claims in days rather than weeks, and its large and growing team based on Sydney’s Northern Beaches.
+FreightSafe solution offered via Fast Courier to protect goods in transit (10/11/2021)
+Fast Courier promotes FreightSafe as an extended‑warranty / transit‑protection option, allowing every consignment booked through the platform to be covered against loss or damage at varying levels. This reflects an earlier stage of FreightSafe’s growth in embedded protection services, broadening its distribution through online freight marketplaces and increasing its exposure to small and medium‑sized shippers using digital booking channels.</t>
+        </is>
+      </c>
+      <c r="D119" s="17" t="inlineStr"/>
+      <c r="E119" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="16" t="inlineStr">
+        <is>
+          <t>FundBase Group</t>
+        </is>
+      </c>
+      <c r="B120" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C120" s="17" t="inlineStr">
+        <is>
+          <t>FundBase to launch platform for retail access to private markets (27/11/2023)
+FundBase Group, the Sydney‑based investment fund infrastructure provider, announced plans to launch a new platform aimed at giving Australian retail investors access to private markets. The initiative expands FundBase Group’s service offering beyond institutional and wholesale managers, positioning the firm to capture growing retail interest in private assets and signalling product expansion and business growth.
+FundBase Group expands into integrated fund infrastructure platform (01/06/2023)
+Originally established to solve internal operational challenges for fund administration and back‑office support, FundBase Group has expanded its model into an integrated fund infrastructure platform supported by proprietary technology. This evolution, highlighted in the firm’s corporate materials, reflects organic growth in client numbers and service breadth, as the company now provides end‑to‑end fund operations and institutional‑grade infrastructure for emerging and established managers across Australia.
+FundBase Group increases national footprint with offices in Sydney, Brisbane and Melbourne (01/03/2023)
+FundBase Group reports a broadened national presence with offices listed in Sydney, Brisbane and Melbourne, demonstrating geographic expansion beyond its original Sydney base. By operating from multiple CBD locations, the firm is strengthening its service coverage for fund managers across Australia, supporting continued client and headcount growth in its fund infrastructure and administration services.</t>
+        </is>
+      </c>
+      <c r="D120" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Announcement of a collaboration with Serena Williams and Reckitt to leverage networks for opportunities.
+[27/04/2026 - 3w] LinkedIn's achievement as the top-cited domain for professional queries indicating its significant impact and growth in AI context.
+[22/04/2026 - 3w] Announcement of leadership changes at LinkedIn, highlighting the growth potential for the company.</t>
+        </is>
+      </c>
+      <c r="E120" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="16" t="inlineStr">
+        <is>
+          <t>FuseWorks (Brisbane, Queensland, Australia)</t>
+        </is>
+      </c>
+      <c r="B121" s="16" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="C121" s="17" t="inlineStr">
+        <is>
+          <t>FuseWorks strengthens client support with dedicated Brisbane-based operations (15/11/2023)
+Through its updated contact and company information, FuseWorks confirms a dedicated Brisbane CBD presence at Level 10, 300 Ann Street, along with structured support hours and centralised client assistance. While not a formal press release, the consolidation of office details and support infrastructure reflects an established and growing software provider investing in local operations to better service an expanding client base of accounting firms.
+FuseWorks highlights Brisbane HQ and Australian-based development team (01/06/2023)
+FuseWorks updated its ‘About Us’ and ‘Meet the Team’ pages to emphasise its Brisbane headquarters and locally developed and hosted software. The expanded team profiles and positioning—“made for accountants by accountants” and “all of our products are designed, developed and hosted in Australia in our Brisbane HQ”—indicate a maturing organisation with an in‑house development and support team, supporting continued product expansion and stronger service capability for accounting firms across Australia.
+FuseWorks showcases client growth through automation case studies (10/08/2022)
+FuseWorks published a series of case studies on its website demonstrating how accounting firms have scaled their operations using FuseWorks products such as FuseDocs and FuseSign. The case studies describe firms reducing manual admin work, cutting processing times, and handling higher client volumes without equivalent staff increases. This content signals ongoing adoption of FuseWorks’ products by accounting practices and underlines the company’s role in enabling clients’ operational growth and cost savings.
+Accountants can lean on technology to improve client relationships (15/03/2021)
+In this sponsored feature on AccountantsDaily, FuseWorks is profiled as a key technology partner helping accounting firms improve client relationships and efficiency. The article highlights FuseWorks’ suite of tools (including digital signing and document automation) as examples of how firms are increasingly adopting specialised software to streamline workflows, free up staff time, and expand value‑adding advisory services. The coverage positions FuseWorks as a growing player in the Australian accounting-tech space that supports firm growth and profitability through automation.</t>
+        </is>
+      </c>
+      <c r="D121" s="17" t="inlineStr">
+        <is>
+          <t>[18/05/2026 - 1d] Celebrating Jackson Brigg's five-year anniversary reflects company growth and employee development.
+[15/05/2026 - 4d] FuseWorks engaged with William Buck at their National Partner Conference to strengthen collaborations.
+[07/05/2026 - 1w] FuseWorks recognized as a Top 5 Best Workplace in Technology 2026, reflecting strong team culture.
+[07/05/2026 - 1w] FuseWorks is hiring a Technical Client Service Specialist to aid in further company growth.
+[05/05/2026 - 2w] The launch of a new FuseSign video highlights positive impacts on client practices due to streamlined signing process.</t>
+        </is>
+      </c>
+      <c r="E121" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fuseworksteam/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="16" t="inlineStr">
+        <is>
+          <t>Fuseco</t>
+        </is>
+      </c>
+      <c r="B122" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C122" s="17" t="inlineStr"/>
+      <c r="D122" s="17" t="inlineStr">
+        <is>
+          <t>[12/05/2026 - 1w] Launch announcement of the ChargeMaster ShockSafe UPS, highlighting its innovative safety features.
+[27/04/2026 - 3w] Announcement of a $3 million upgrade project supported by Fuseco, showcasing their involvement in renewable energy advancements.
+[21/04/2026 - 4w] Hiring announcement for a new customer service role, indicating team growth and expansion.</t>
+        </is>
+      </c>
+      <c r="E122" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fuseco-pty-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="16" t="inlineStr">
+        <is>
+          <t>GCG Health Safety Hygiene</t>
+        </is>
+      </c>
+      <c r="B123" s="16" t="inlineStr">
+        <is>
+          <t>Perth</t>
+        </is>
+      </c>
+      <c r="C123" s="17" t="inlineStr">
+        <is>
+          <t>GCG recognised as a leading national WHS and occupational hygiene specialist (10/11/2022)
+In updated corporate materials, GCG Health Safety Hygiene described itself as one of Australia’s leading workplace health and occupational hygiene specialists with over 20 years of operation, reflecting long‑term growth from a small consultancy to a national firm. The company’s expanded geographic footprint and multi‑industry client base, ranging from aerospace to mining to water and energy, illustrate its sustained revenue and capability growth in the management consulting segment of WHS and occupational hygiene.
+GCG strengthens leadership team to support national WHS consulting growth (22/07/2021)
+GCG Health Safety Hygiene publicised additions and promotions within its leadership team, building depth in national management to support a growing portfolio of WHS and occupational hygiene contracts. The refreshed leadership structure was positioned as a key step in scaling delivery across sectors such as mining, water, energy and manufacturing and in supporting continued expansion from its offices including Perth and New South Wales.
+GCG expands capabilities and wins national recognition through growth in occupational hygiene and WHS services (15/03/2019)
+Through a series of internal announcements and case studies, GCG Health Safety Hygiene highlighted expansion in its occupational hygiene and WHS service lines, including larger project engagements in mining, energy and infrastructure. The company reported an increase in senior consultants and project managers across Australia and showcased recognition from major clients for its role in improving workplace exposure monitoring and safety performance, indicating sustained business and headcount growth.
+GCG appoints first Federal Safety Officers to support national WHS growth (28/09/2016)
+GCG Health Safety Hygiene announced the appointment of its first Federal Safety Officers, expanding its capability to support clients working under the Australian Government Building and Construction WHS Accreditation Scheme. The appointments reflect growing national demand for GCG’s specialist WHS and occupational hygiene services and strengthen its position as a key provider to construction and infrastructure projects across Australia.</t>
+        </is>
+      </c>
+      <c r="D123" s="17" t="inlineStr">
+        <is>
+          <t>[13/05/2026 - 6d] Celebrating team members' five-year milestones, indicating employee retention and recognition of contributions.
+[22/04/2026 - 3w] GCG is a finalist in the 2026 Hunter Safety Awards for their Exposi Hygiene Management System, highlighting recognition for innovation.</t>
+        </is>
+      </c>
+      <c r="E123" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/gcgaust/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="16" t="inlineStr">
+        <is>
+          <t>GPC Electronics (138 Blaikie Road, Jamisontown, NSW, 2750, AU)</t>
+        </is>
+      </c>
+      <c r="B124" s="16" t="inlineStr">
+        <is>
+          <t>New South Wales</t>
+        </is>
+      </c>
+      <c r="C124" s="17" t="inlineStr">
+        <is>
+          <t>GPC Electronics continues to scale as one of Australasia’s largest contract manufacturers (10/06/2024)
+A company overview on GPC Electronics’ own site and syndicated business directories describes the Jamisontown-based business as one of Australasia’s largest contract manufacturers, with three manufacturing locations in Sydney (NSW), Christchurch (NZ) and Shenzhen (China), and most production exported to more than 40 countries. The profile notes ongoing expansion of production lines and a workforce of roughly 279 employees across the group, along with a revenue base approaching $60 million. These details indicate sustained growth in scale, exports and group-wide employment, with the NSW headquarters as the central hub of operations.
+AUKUS Connect highlights GPC Electronics’ expanded defence-related manufacturing capability (03/08/2023)
+An AUKUS Forum profile on AUKUS Connect features GPC Electronics, founded in 1985 by Christopher Janssen, noting that the NSW-headquartered firm now operates nine state-of-the-art electronics production and testing lines across its network. The piece emphasizes GPC’s role in supplying complex electronics into defence and allied sectors and its focus on sovereign manufacturing capability within the AUKUS framework. This coverage points to the company’s scaling of high‑reliability production capacity and its strategic alignment with growing defence and security-related demand, reflecting both capability and market growth anchored from its Jamisontown headquarters.
+Carbonix and GPC Electronics partner to advance Australian drone sector (09/05/2023)
+Sydney-based Carbonix and GPC Electronics Group announced a partnership to enhance sovereign capability in Australia’s drone and UAV sector. Under the collaboration, GPC Electronics’ Jamisontown-based advanced electronics manufacturing will support Carbonix’s production of sophisticated drone systems, bringing high‑reliability local manufacturing into a segment that often relies on overseas supply chains. The partnership signals GPC’s strategic move into the growing UAV/defence-adjacent market, leveraging its existing export-grade manufacturing capabilities and reinforcing its role as a key domestic electronics manufacturing partner for high-technology Australian companies.
+Penrith manufacturer has global reach (19/01/2022)
+Penrith City Council profiled GPC Electronics as one of Australasia’s largest contract electronics manufacturers, highlighting that it has grown since its 1985 founding to serve global giants such as Toshiba, Nortel, Ericsson, Siemens, Daikin, Johnson Controls, Schneider, Philips and numerous Australian start-ups. The article notes that GPC’s Jamisontown headquarters now employs around 150 people, manufactures products for communications, industrial, agricultural, medical, automotive and defence industries, and exports customers’ products to roughly 40 countries. The company has expanded its footprint with additional facilities in China and New Zealand, underscoring sustained international growth and diversification of its customer base and end markets.
+Thought Leadership: Insights from GPC Electronics’ Managing Director (15/11/2020)
+In a thought-leadership interview hosted by Hawker Richardson, Managing Director Christopher Janssen describes how GPC Electronics, founded in 1985 in New South Wales, has evolved into a global provider of electronics manufacturing services. He outlines the company’s growth from a local contract manufacturer to an exporter serving over 40 countries, supported by facilities in Australia, New Zealand and China. The discussion focuses on scaling advanced manufacturing lines, investing in surface-mount technology and end-to-end EMS capabilities, and positioning the Jamisontown headquarters as the core of a broader regional network—illustrating sustained operational and geographic growth tied directly to its NSW base.</t>
+        </is>
+      </c>
+      <c r="D124" s="17" t="inlineStr"/>
+      <c r="E124" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/gpc-electronics/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="16" t="inlineStr">
+        <is>
+          <t>Genesis Research Services (Broadmeadow, New South Wales, Australia)</t>
+        </is>
+      </c>
+      <c r="B125" s="16" t="inlineStr">
+        <is>
+          <t>New South Wales</t>
+        </is>
+      </c>
+      <c r="C125" s="17" t="inlineStr">
+        <is>
+          <t>Genesis Research Services earns NSW Health Clinical Trials Quality Recognition Scheme (QRS) status (13/10/2025)
+Genesis Research Services has been officially recognised by NSW Health under the Clinical Trials Quality Recognition Scheme (QRS), becoming only the second clinical trials site to receive this status. The recognition highlights the organisation’s strength in clinical and medical governance, quality processes, risk management, research team capability, and emergency response readiness, reinforcing its position as a high‑quality independent clinical research site.
+Genesis Research Services reports team expansion with new hires over the past 12 months (01/09/2025)
+Profile information on Genesis Research Services indicates that the organisation is expanding and has recently hired additional staff over the previous 12 months. The added team members support its clinical trial operations and related services, signalling ongoing growth in capability and activity at its Broadmeadow, NSW site.
+Genesis Research Services moves into larger, purpose-designed clinical trials facility in Broadmeadow (15/01/2025)
+Genesis Research Services announced that it has relocated to a newly renovated, purpose-designed clinical trials facility at Ground Floor, 239/245 Denison Street, Broadmeadow NSW 2292, directly across from its previous site. The new space offers a more spacious and modern environment with dedicated participant parking and improved access, supporting expanded clinical trial activity and a better experience for study participants.</t>
+        </is>
+      </c>
+      <c r="D125" s="17" t="inlineStr"/>
+      <c r="E125" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/genesis-research-services-pty-ltd/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="16" t="inlineStr">
+        <is>
+          <t>Genomics For Life Pty Ltd (Brisbane, QLD, Australia)</t>
+        </is>
+      </c>
+      <c r="B126" s="16" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="C126" s="17" t="inlineStr">
+        <is>
+          <t>Genomics For Life expands clinical and oncology genomic testing menu to over 3,000 genes (01/03/2024)
+Genomics For Life, a NATA‑accredited private pathology laboratory based in Milton, Brisbane, has expanded its clinical and oncology genomic testing range to cover more than 3,000 genes associated with cancer and inherited disease. The broadened menu, highlighted in updated service information for clinicians, positions the lab as having one of the largest genetic testing options of any laboratory in Australia and reflects continued investment in next‑generation sequencing capabilities and assay development.
+Brisbane-based Genomics For Life highlighted as leading private cancer genomics laboratory in Australia (15/11/2023)
+Industry and member communications in the Australian genomics sector reference Genomics For Life Pty Ltd, headquartered in Milton, Brisbane, as a key private pathology provider specialising in cancer genomics and inherited disease testing. The laboratory’s NATA accreditation to ISO 15189 standards and its positioning among Australia’s major oncology genomics services indicate reputational growth and consolidation as a specialist provider in precision oncology and hereditary cancer diagnostics.</t>
+        </is>
+      </c>
+      <c r="D126" s="17" t="inlineStr"/>
+      <c r="E126" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/genomics-for-life/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="16" t="inlineStr">
+        <is>
+          <t>GoodHuman (Sydney, New South Wales, Australia)</t>
+        </is>
+      </c>
+      <c r="B127" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C127" s="17" t="inlineStr">
+        <is>
+          <t>GoodHuman launches all‑in‑one NDIS service delivery platform for human services providers (15/03/2023)
+GoodHuman, the Sydney‑based human services software company, announced major product updates to its purpose‑built NDIS service delivery platform, integrating workforce, customer and billing management into a single system. The company positions the enhanced platform as the only all‑in‑one solution specifically designed for the human services sector, aiming to help providers scale, streamline operations and deliver greater impact. The breadth of new functionality and repositioning toward larger providers indicate product‑led growth and stronger market traction in Australia’s disability and community services markets.
+GoodHuman strengthens position as a customer success engine for NDIS providers (10/08/2022)
+Startup profiles describe GoodHuman as a fast‑growing Melbourne‑ and Sydney‑linked software startup providing a customer success engine for NDIS service providers. The GoodHuman app enables participants to discover and connect with local support services, while providers use the platform for CRM and case management, rostering and scheduling, mobile workforce management, and instant invoicing and billing. The broadened feature set and emphasis on helping providers grow their business and streamline processes reflect ongoing platform development and an expanding customer base in the NDIS ecosystem.
+GoodHuman highlights growing enterprise focus for human services organisations (01/06/2022)
+Through its ‘GoodHuman for Enterprise’ offering, the company signals a strategic move up‑market toward large, complex human services organisations. The enterprise solution emphasises flexible, scalable features that can evolve with providers as they grow, connecting NDIS participants, rosters, bookings and billing at scale. This enterprise positioning suggests that GoodHuman is targeting larger contracts and more sophisticated providers, indicating a growth strategy beyond smaller organisations and individual support networks.</t>
+        </is>
+      </c>
+      <c r="D127" s="17" t="inlineStr"/>
+      <c r="E127" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/goodhuman/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="16" t="inlineStr">
+        <is>
+          <t>GreenBe</t>
+        </is>
+      </c>
+      <c r="B128" s="16" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="C128" s="17" t="inlineStr"/>
+      <c r="D128" s="17" t="inlineStr">
+        <is>
+          <t>[07/05/2026 - 1w] Discusses a collaboration with Serena Williams and Reckitt, focusing on leveraging networks for business opportunities.
+[27/04/2026 - 3w] Highlights LinkedIn's status as a leading domain in AI search engines, suggesting market expansion and increased visibility.
+[24/04/2026 - 3w] Announces Fernando Mendoza's official role confirmation, indicating a new hire that suggests growth opportunities.
+[22/04/2026 - 3w] Congratulates new leadership appointments at LinkedIn, indicating team growth and strategic positioning for future opportunities.</t>
+        </is>
+      </c>
+      <c r="E128" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/linkedin/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="16" t="inlineStr">
+        <is>
+          <t>Gullotta Orthodontics (Dr Nino Gullotta), Southport, Gold Coast, QLD, Australia</t>
+        </is>
+      </c>
+      <c r="B129" s="16" t="inlineStr">
+        <is>
+          <t>Gold Coast</t>
+        </is>
+      </c>
+      <c r="C129" s="17" t="inlineStr">
+        <is>
+          <t>Gullotta Orthodontics Awarded Invisalign Diamond Provider Status (01/07/2023)
+Gullotta Orthodontics, led by Gold Coast orthodontist Dr Nino Gullotta, has been awarded Invisalign Diamond Provider status, reflecting a high volume of successful Invisalign cases and strong clinical expertise. This recognition positions the Southport-based clinic among the top tiers of Invisalign providers and indicates sustained patient growth and treatment demand.
+Gullotta Orthodontics Recognised as One of the Top 3 Orthodontists on the Gold Coast (15/03/2022)
+Review platform ThreeBestRated lists Dr Nino Gullotta and Gullotta Orthodontics as one of the top three orthodontic practices on the Gold Coast. The recognition is based on factors such as reputation, reviews, service quality, and patient satisfaction, highlighting the clinic’s strong market position and ongoing growth in its patient base.
+Gullotta Orthodontics Marks Over 35 Years of Specialist Orthodontic Practice on the Gold Coast (01/06/2021)
+Gullotta Orthodontics celebrates more than 35 years since its establishment in 1987 by founder and director Dr Nino Gullotta. Over this period, the Southport practice has treated thousands of patients and grown into one of the Gold Coast’s most experienced and highly rated orthodontic providers, indicating long-term business stability and sustained demand for its services.</t>
+        </is>
+      </c>
+      <c r="D129" s="17" t="inlineStr"/>
+      <c r="E129" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/gullotta-orthodontics/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="16" t="inlineStr">
+        <is>
+          <t>Hardcat Pty Ltd</t>
+        </is>
+      </c>
+      <c r="B130" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C130" s="17" t="inlineStr">
+        <is>
+          <t>Hardcat extends global footprint via new Indian partnership with Yotta (01/02/2023)
+The Victorian Government’s Global Victoria program profiled Hardcat as a world leader in asset and evidence management and highlighted its expansion into India through a partnership with Yotta of the Hiranandani Group. The partnership builds on Hardcat’s existing global presence, which already includes wholly owned subsidiaries in the USA, UK and Africa, and a customer base featuring major corporates and public-sector agencies. This signals ongoing international growth for the Melbourne-based software company.
+Yotta partners with Melbourne-based Hardcat to launch Lebosi enterprise asset management platform in India (05/01/2023)
+Yotta Data Services (formerly Yotta Infrastructure) announced an exclusive partnership with Hardcat Pty Ltd of Melbourne to introduce Hardcat’s Lebosi enterprise asset management solution to the Indian market. The collaboration leverages Yotta’s data centre and service delivery capabilities to offer Hardcat’s cloud-based, lifecycle asset management platform to Indian enterprise and government customers, expanding Hardcat’s geographic reach and customer base in a large new market.
+Hardcat positions cloud-based asset and inventory platform for multi-industry growth (01/06/2022)
+Company profile data indicates that Hardcat has evolved into a cloud-based asset, tools and equipment tracking platform serving defence, police, emergency services, aged care, banking, mining and telecom sectors. The suite has expanded with multiple add-on modules such as preventive maintenance, depreciation, stock, procurement and help desk, reflecting product-line growth and broader industry adoption. This positioning underlines Hardcat’s strategy of scaling recurring SaaS revenue across diverse verticals.
+New version of Hardcat software supports strategic customer growth with modern technologies (01/09/2019)
+An industry article described a new version of Hardcat’s asset management software that incorporates evolving technology trends including bar-code scanning and mobile handheld devices. The release demonstrates ongoing product innovation designed to support customers’ strategic growth and operational efficiency, reinforcing Hardcat’s position as a long-standing provider adapting its platform to modern enterprise requirements.
+Hardcat prepares major new release and Next Gen system generator platform (01/01/2009)
+In a Q&amp;A with Managing Director Dan Drum, Hardcat outlined plans for a major software release in January 2009 featuring multilingual web support, user-selectable web templates, and GPS/GIS capabilities, along with a forthcoming ‘Hardcat Next Gen’ product described as a sophisticated system generator four years in development. These releases indicate substantial R&amp;D investment aimed at expanding functionality and supporting future growth.</t>
+        </is>
+      </c>
+      <c r="D130" s="17" t="inlineStr">
+        <is>
+          <t>[29/04/2026 - 2w] Announcement of a collaboration between Hardcat and Zebra to enhance asset intelligence solutions.
+[22/04/2026 - 3w] Discussion on the capabilities of Hardcat Lebosi EAM in improving asset management operations for organizations.</t>
+        </is>
+      </c>
+      <c r="E130" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/hardcat/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="16" t="inlineStr">
+        <is>
+          <t>Hawke's Bay Orthodontics</t>
+        </is>
+      </c>
+      <c r="B131" s="16" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C131" s="17" t="inlineStr">
+        <is>
+          <t>Hawke's Bay Orthodontics highlights expanded treatment range for children and adults (15/03/2024)
+Hawke's Bay Orthodontics in Havelock North has been promoting its broadened suite of orthodontic services, including metal and clear ceramic braces, Invisalign, removable plates and functional appliances. The practice emphasises tailored treatment plans for both children and adults, signalling ongoing investment in modern orthodontic options and service capability for the Hawke's Bay community.
+Regional feature showcases Hawke's Bay Orthodontics as one of three key specialist practices in Hawke's Bay (10/02/2023)
+Orthodontics New Zealand’s directory of Hawke’s Bay specialists lists Hawke's Bay Orthodontics among three main specialist orthodontic practices serving the region. The listing underscores the practice’s established position and continued role in meeting growing demand for specialist orthodontic care across Napier, Hastings, Havelock North and surrounding towns.
+Practice update notes collaboration with specialist orthodontists across Hawke's Bay and Gisborne (20/11/2022)
+Information on partner practice sites indicates that Hawke’s Bay Orthodontics works in collaboration with specialist orthodontists such as Dr Andrew Parton, who splits his time between his Taradale practice and Hawke’s Bay Orthodontics in Havelock North. This shared-specialist model reflects a growth‑oriented approach to increasing specialist availability and service coverage across the wider region.</t>
+        </is>
+      </c>
+      <c r="D131" s="17" t="inlineStr"/>
+      <c r="E131" s="16" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="16" t="inlineStr">
+        <is>
+          <t>Hearth Support Services (Melbourne, Australia)</t>
+        </is>
+      </c>
+      <c r="B132" s="16" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="C132" s="17" t="inlineStr">
+        <is>
+          <t>Expansion of Support Worker and Allied Health Teams Across Melbourne and Victoria (15/03/2023)
+Hearth Support Services has continued hiring extensively for Support Workers and allied health professionals, signalling ongoing operational expansion in Melbourne and across Victoria. The organisation promotes multiple open roles and clear internal career pathways (including Relationship Manager positions and Allied Health career tracks), indicating both workforce growth and a maturing organisational structure to support more NDIS participants in home and community settings.
+Hearth Support Services Turns Five and Celebrates Rapid Growth Since 2017 (07/04/2022)
+Hearth Support Services marked its fifth anniversary by highlighting “enormous change” and rapid expansion since its inception in 2017. The Melbourne-based NDIS provider reported significant growth in client numbers and service offerings, including support worker services, allied health, and broader NDIS registration groups. The milestone piece emphasises that the organisation has scaled its operations while maintaining a person-centred model and building a larger multidisciplinary team.
+Hearth Support Services Broadens NDIS-Registered Service Categories (10/08/2021)
+Hearth Support Services Pty Ltd is listed by the NDIS Quality and Safeguards Commission as an approved provider across a wide range of registration groups, including Assist Personal Activities High, Daily Tasks/Shared Living, Community Nursing Care, Development-Life Skills, and more. This breadth of approved categories reflects a strategic expansion from basic support worker services into higher-intensity care, community participation, life skills development, and employment-related supports, allowing the company to serve a larger and more diverse participant base.
+Service Offering Expansion: Comprehensive Home and Community Supports for NDIS Participants (01/09/2020)
+Hearth Support Services has expanded its Melbourne-based service offering to cover a comprehensive suite of home and community supports for NDIS participants. These include daily living assistance, high-intensity care and complex medical support, post-hospital discharge support, independent living skills training (meals, household duties, travel skills), manual handling and mobility assistance, behaviour support plan implementation, and specialised training in collaboration with allied health professionals. The diversified service mix positions Hearth to capture broader NDIS demand and indicates sustained service-line growth.</t>
+        </is>
+      </c>
+      <c r="D132" s="17" t="inlineStr">
+        <is>
+          <t>[15/05/2026 - 4d] Announcement of a job opening for an experienced Occupational Therapist, indicating team growth in Allied Health practice.
+[12/05/2026 - 1w] Details about growth at Hearth, including job opportunities and the positive impact of their housing solutions in healthcare and disability services.
+[07/05/2026 - 1w] Job opportunity at the head office in Glen Iris that combines administration with passion for healthcare, indicating growth and need for support staff.
+[01/05/2026 - 2w] Mention of increased requirements in the Allied Health practice due to innovative housing solutions, indicating business expansion.</t>
+        </is>
+      </c>
+      <c r="E132" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/hearth-personal-care-services/posts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="16" t="inlineStr">
+        <is>
+          <t>Hekate (New Zealand, e-commerce retailer)</t>
+        </is>
+      </c>
+      <c r="B133" s="16" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C133" s="17" t="inlineStr"/>
+      <c r="D133" s="17" t="inlineStr"/>
+      <c r="E133" s="16" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="16" t="inlineStr">
+        <is>
+          <t>energyOS</t>
+        </is>
+      </c>
+      <c r="B134" s="16" t="inlineStr">
+        <is>
+          <t>Perth</t>
+        </is>
+      </c>
+      <c r="C134" s="17" t="inlineStr">
+        <is>
+          <t>Electrifying SaaS growth through full-service support | Case study (01/01/2024)
+A case study featuring energyOS highlights the company as an Australian SaaS platform serving electricity and gas utilities, with CEO Stephen Kubicki discussing support for the company’s growth and expansion as it helps utilities respond to the energy transition.
+Client Story: energyOS (01/01/2024)
+RSM’s client story on energyOS says CEO Stephen Kubicki has ambitious plans to grow the company and expand its presence in the global market, indicating business expansion and scaling activity for the Perth-based software firm.</t>
+        </is>
+      </c>
+      <c r="D134" s="17" t="inlineStr"/>
+      <c r="E134" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/energyossolutions/posts/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>